<commit_message>
refinando a tradução com claude opus 4.6
</commit_message>
<xml_diff>
--- a/translations Dance2Dance.xlsx
+++ b/translations Dance2Dance.xlsx
@@ -591,7 +591,7 @@
       </c>
       <c r="E2" s="5" t="inlineStr">
         <is>
-          <t>See Schedule</t>
+          <t>View Schedule</t>
         </is>
       </c>
       <c r="F2" s="5" t="inlineStr">
@@ -604,7 +604,11 @@
           <t>Completo (3 idiomas)</t>
         </is>
       </c>
-      <c r="H2" s="5" t="inlineStr"/>
+      <c r="H2" s="5" t="inlineStr">
+        <is>
+          <t>[EN: Standard UI convention in English.]</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="7" t="n">
@@ -1059,12 +1063,12 @@
       </c>
       <c r="E15" s="10" t="inlineStr">
         <is>
-          <t>Every body carries a dance it hasn't yet dared to step into. These workshops are the space where movement, presence and expression bring it to light.</t>
+          <t>Every body holds a dance it hasn't yet dared to release. These workshops are a space where movement, presence, and expression bring it to light.</t>
         </is>
       </c>
       <c r="F15" s="10" t="inlineStr">
         <is>
-          <t>Hver kropp bærer en dans den ennå ikke har våget å slippe ut. Disse verkstedene er rommet der bevegelse, tilstedeværelse og uttrykk bringer den frem i lyset.</t>
+          <t>Hver kropp bærer på en dans den ennå ikke har våget å slippe fri. Disse workshopene er rommet hvor bevegelse, tilstedeværelse og uttrykk bringer den frem i lyset.</t>
         </is>
       </c>
       <c r="G15" s="11" t="inlineStr">
@@ -1072,7 +1076,11 @@
           <t>Completo (3 idiomas)</t>
         </is>
       </c>
-      <c r="H15" s="10" t="inlineStr"/>
+      <c r="H15" s="10" t="inlineStr">
+        <is>
+          <t>[EN: More poetic and natural phrasing.] | [NO: Changed to 'bærer på' (more idiomatic), 'slippe fri' (more poetic), and 'workshopene' (more common than 'verkstedene' in this context).]</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
@@ -1095,12 +1103,12 @@
       </c>
       <c r="E16" s="5" t="inlineStr">
         <is>
-          <t>Conscious movement practices that broaden perception, stimulate body reorganization and transform the way we inhabit the body.</t>
+          <t>Conscious movement practices that expand perception, encourage bodily reorganization, and transform how we inhabit our bodies.</t>
         </is>
       </c>
       <c r="F16" s="5" t="inlineStr">
         <is>
-          <t>Bevisste bevegelsespraksiser som utvider oppfatningen, stimulerer kroppslig omorganisering og forvandler måten vi bor i kroppen på.</t>
+          <t>Bevisste bevegelsespraksiser som utvider sanseopplevelsen, stimulerer kroppslig omorganisering og forvandler måten vi er i egen kropp på.</t>
         </is>
       </c>
       <c r="G16" s="6" t="inlineStr">
@@ -1108,7 +1116,11 @@
           <t>Completo (3 idiomas)</t>
         </is>
       </c>
-      <c r="H16" s="5" t="inlineStr"/>
+      <c r="H16" s="5" t="inlineStr">
+        <is>
+          <t>[EN: Improves flow and uses more natural English collocations.] | [NO: 'oppfatningen' means opinion/understanding; 'sanseopplevelsen' is correct for sensory perception. 'er i egen kropp på' sounds much more natural than 'bor i kroppen på'.]</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="7" t="n">
@@ -1131,7 +1143,7 @@
       </c>
       <c r="E17" s="10" t="inlineStr">
         <is>
-          <t>Community projects that cross streets and neighborhoods, weaving ties, creating bonds and transforming.</t>
+          <t>Community projects that reach across streets and neighborhoods—weaving connections, building bonds, and sparking transformation.</t>
         </is>
       </c>
       <c r="F17" s="10" t="inlineStr">
@@ -1144,7 +1156,11 @@
           <t>Completo (3 idiomas)</t>
         </is>
       </c>
-      <c r="H17" s="10" t="inlineStr"/>
+      <c r="H17" s="10" t="inlineStr">
+        <is>
+          <t>[EN: More natural, dynamic, and poetic verbs.]</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="n">
@@ -1167,7 +1183,7 @@
       </c>
       <c r="E18" s="5" t="inlineStr">
         <is>
-          <t>SEE OUR SCHEDULE</t>
+          <t>EXPLORE OUR SCHEDULE</t>
         </is>
       </c>
       <c r="F18" s="5" t="inlineStr">
@@ -1180,7 +1196,11 @@
           <t>Completo (3 idiomas)</t>
         </is>
       </c>
-      <c r="H18" s="5" t="inlineStr"/>
+      <c r="H18" s="5" t="inlineStr">
+        <is>
+          <t>[EN: More inviting and warm call-to-action.]</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="7" t="n">
@@ -1311,7 +1331,7 @@
       </c>
       <c r="E22" s="5" t="inlineStr">
         <is>
-          <t>Add to Instructor Calendar (Google Calendar)</t>
+          <t>Add to Instructor's Calendar (Google Calendar)</t>
         </is>
       </c>
       <c r="F22" s="5" t="inlineStr">
@@ -1324,7 +1344,11 @@
           <t>Completo (3 idiomas)</t>
         </is>
       </c>
-      <c r="H22" s="5" t="inlineStr"/>
+      <c r="H22" s="5" t="inlineStr">
+        <is>
+          <t>[EN: Grammatical correction for possessive form.]</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="7" t="n">
@@ -1383,7 +1407,7 @@
       </c>
       <c r="E24" s="5" t="inlineStr">
         <is>
-          <t>Auto Generate Schedule</t>
+          <t>Generate Schedule Summary</t>
         </is>
       </c>
       <c r="F24" s="5" t="inlineStr">
@@ -1396,7 +1420,11 @@
           <t>Completo (3 idiomas)</t>
         </is>
       </c>
-      <c r="H24" s="5" t="inlineStr"/>
+      <c r="H24" s="5" t="inlineStr">
+        <is>
+          <t>[EN: More accurate translation of Resumo da Programação.]</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="7" t="n">
@@ -2175,7 +2203,7 @@
       </c>
       <c r="E46" s="5" t="inlineStr">
         <is>
-          <t>End date cannot be prior to start date.</t>
+          <t>End date cannot be before the start date.</t>
         </is>
       </c>
       <c r="F46" s="5" t="inlineStr">
@@ -2188,7 +2216,11 @@
           <t>Completo (3 idiomas)</t>
         </is>
       </c>
-      <c r="H46" s="5" t="inlineStr"/>
+      <c r="H46" s="5" t="inlineStr">
+        <is>
+          <t>[EN: More natural phrasing for UI error messages.]</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="7" t="n">
@@ -6212,7 +6244,7 @@
       </c>
       <c r="F158" s="5" t="inlineStr">
         <is>
-          <t>Flest Kurs Gjennomført</t>
+          <t>Flest gjennomførte kurs</t>
         </is>
       </c>
       <c r="G158" s="6" t="inlineStr">
@@ -6220,7 +6252,11 @@
           <t>Completo (3 idiomas)</t>
         </is>
       </c>
-      <c r="H158" s="5" t="inlineStr"/>
+      <c r="H158" s="5" t="inlineStr">
+        <is>
+          <t>[NO: More natural Norwegian word order.]</t>
+        </is>
+      </c>
     </row>
     <row r="159">
       <c r="A159" s="7" t="n">
@@ -6747,7 +6783,7 @@
       </c>
       <c r="E173" s="10" t="inlineStr">
         <is>
-          <t>Follow our upcoming dates for workshops, regular sessions, and experiences from Be The Dance and Biostretch.</t>
+          <t>Stay updated on our upcoming workshops, regular sessions, and immersive experiences by Be The Dance and Biostretch.</t>
         </is>
       </c>
       <c r="F173" s="10" t="inlineStr">
@@ -6760,7 +6796,11 @@
           <t>Completo (3 idiomas)</t>
         </is>
       </c>
-      <c r="H173" s="10" t="inlineStr"/>
+      <c r="H173" s="10" t="inlineStr">
+        <is>
+          <t>[EN: More engaging marketing tone.]</t>
+        </is>
+      </c>
     </row>
     <row r="174">
       <c r="A174" s="2" t="n">
@@ -8871,7 +8911,7 @@
       </c>
       <c r="E232" s="5" t="inlineStr">
         <is>
-          <t>Tell us briefly about your dance experience...</t>
+          <t>Tell us briefly about your experience...</t>
         </is>
       </c>
       <c r="F232" s="5" t="inlineStr">
@@ -8884,7 +8924,11 @@
           <t>Completo (3 idiomas)</t>
         </is>
       </c>
-      <c r="H232" s="5" t="inlineStr"/>
+      <c r="H232" s="5" t="inlineStr">
+        <is>
+          <t>[EN: The Portuguese original doesn't limit it to dance in the placeholder, it keeps it open.]</t>
+        </is>
+      </c>
     </row>
     <row r="233">
       <c r="A233" s="7" t="n">
@@ -10347,7 +10391,7 @@
       </c>
       <c r="E273" s="10" t="inlineStr">
         <is>
-          <t>There is a possibility of dance in every body.</t>
+          <t>A possibility of dance exists within every body.</t>
         </is>
       </c>
       <c r="F273" s="10" t="inlineStr">
@@ -10360,7 +10404,11 @@
           <t>Completo (3 idiomas)</t>
         </is>
       </c>
-      <c r="H273" s="10" t="inlineStr"/>
+      <c r="H273" s="10" t="inlineStr">
+        <is>
+          <t>[EN: Slightly more poetic and fluid sentence structure.]</t>
+        </is>
+      </c>
     </row>
     <row r="274">
       <c r="A274" s="2" t="n">
@@ -10923,7 +10971,7 @@
       </c>
       <c r="E289" s="10" t="inlineStr">
         <is>
-          <t>It needs to be permitted.</t>
+          <t>It needs to be allowed.</t>
         </is>
       </c>
       <c r="F289" s="10" t="inlineStr">
@@ -10936,7 +10984,11 @@
           <t>Completo (3 idiomas)</t>
         </is>
       </c>
-      <c r="H289" s="10" t="inlineStr"/>
+      <c r="H289" s="10" t="inlineStr">
+        <is>
+          <t>[EN: Permitted sounds bureaucratic. Allowed fits the artistic tone much better.]</t>
+        </is>
+      </c>
     </row>
     <row r="290">
       <c r="A290" s="2" t="n">
@@ -10995,12 +11047,12 @@
       </c>
       <c r="E291" s="10" t="inlineStr">
         <is>
-          <t>Each workshop explores a territory.</t>
+          <t>Each workshop explores new territory.</t>
         </is>
       </c>
       <c r="F291" s="10" t="inlineStr">
         <is>
-          <t>Hvert workshop utforsker et territorium.</t>
+          <t>Hver workshop utforsker et landskap.</t>
         </is>
       </c>
       <c r="G291" s="11" t="inlineStr">
@@ -11008,7 +11060,11 @@
           <t>Completo (3 idiomas)</t>
         </is>
       </c>
-      <c r="H291" s="10" t="inlineStr"/>
+      <c r="H291" s="10" t="inlineStr">
+        <is>
+          <t>[EN: More idiomatic expression in English.] | [NO: 'workshop' is common gender (en workshop, hver workshop). 'landskap' is more poetic and fitting than 'territorium'.]</t>
+        </is>
+      </c>
     </row>
     <row r="292">
       <c r="A292" s="2" t="n">
@@ -11067,7 +11123,7 @@
       </c>
       <c r="E293" s="10" t="inlineStr">
         <is>
-          <t>Your body already knows what is tense.</t>
+          <t>Your body already knows where it holds tension.</t>
         </is>
       </c>
       <c r="F293" s="10" t="inlineStr">
@@ -11080,7 +11136,11 @@
           <t>Completo (3 idiomas)</t>
         </is>
       </c>
-      <c r="H293" s="10" t="inlineStr"/>
+      <c r="H293" s="10" t="inlineStr">
+        <is>
+          <t>[EN: More natural phrasing in English bodywork contexts.]</t>
+        </is>
+      </c>
     </row>
     <row r="294">
       <c r="A294" s="2" t="n">
@@ -11247,7 +11307,7 @@
       </c>
       <c r="E298" s="5" t="inlineStr">
         <is>
-          <t>Simple movements. Precise attention.</t>
+          <t>Simple movements. Focused attention.</t>
         </is>
       </c>
       <c r="F298" s="5" t="inlineStr">
@@ -11260,7 +11320,11 @@
           <t>Completo (3 idiomas)</t>
         </is>
       </c>
-      <c r="H298" s="5" t="inlineStr"/>
+      <c r="H298" s="5" t="inlineStr">
+        <is>
+          <t>[EN: Focused attention is a more common collocation in mindful movement.]</t>
+        </is>
+      </c>
     </row>
     <row r="299">
       <c r="A299" s="7" t="n">
@@ -11283,7 +11347,7 @@
       </c>
       <c r="E299" s="10" t="inlineStr">
         <is>
-          <t>Biostretch uses the most accessible tool there is, your attention, to transform how the body organizes itself.</t>
+          <t>Biostretch uses the most accessible tool you have—your attention—to transform how your body organizes itself.</t>
         </is>
       </c>
       <c r="F299" s="10" t="inlineStr">
@@ -11296,7 +11360,11 @@
           <t>Completo (3 idiomas)</t>
         </is>
       </c>
-      <c r="H299" s="10" t="inlineStr"/>
+      <c r="H299" s="10" t="inlineStr">
+        <is>
+          <t>[EN: More direct, conversational, and engaging.]</t>
+        </is>
+      </c>
     </row>
     <row r="300">
       <c r="A300" s="2" t="n">
@@ -11900,7 +11968,7 @@
       </c>
       <c r="F316" s="5" t="inlineStr">
         <is>
-          <t>Hvert workshop jobber med ett lag.</t>
+          <t>Hver workshop jobber med ett lag.</t>
         </is>
       </c>
       <c r="G316" s="6" t="inlineStr">
@@ -11908,7 +11976,11 @@
           <t>Completo (3 idiomas)</t>
         </is>
       </c>
-      <c r="H316" s="5" t="inlineStr"/>
+      <c r="H316" s="5" t="inlineStr">
+        <is>
+          <t>[NO: 'Workshop' is masculine in Norwegian, so it should be 'Hver', not 'Hvert'.]</t>
+        </is>
+      </c>
     </row>
     <row r="317">
       <c r="A317" s="7" t="n">
@@ -12476,7 +12548,7 @@
       </c>
       <c r="F332" s="5" t="inlineStr">
         <is>
-          <t>Ta kontakt for å skreddersy en samling tilpasset din organisasjon.</t>
+          <t>Ta kontakt for å skreddersy et opplegg tilpasset din organisasjon.</t>
         </is>
       </c>
       <c r="G332" s="6" t="inlineStr">
@@ -12484,7 +12556,11 @@
           <t>Completo (3 idiomas)</t>
         </is>
       </c>
-      <c r="H332" s="5" t="inlineStr"/>
+      <c r="H332" s="5" t="inlineStr">
+        <is>
+          <t>[NO: 'Opplegg' (program/setup) is more natural here than 'samling' (gathering) for translating 'proposta' (proposal).]</t>
+        </is>
+      </c>
     </row>
     <row r="333">
       <c r="A333" s="7" t="n">
@@ -14343,7 +14419,7 @@
       </c>
       <c r="E384" s="5" t="inlineStr">
         <is>
-          <t>A space for meeting, movement, and social transformation through dance art and bodily well-being.</t>
+          <t>A space for connection, movement, and social transformation through the art of dance and physical well-being.</t>
         </is>
       </c>
       <c r="F384" s="5" t="inlineStr">
@@ -14356,7 +14432,11 @@
           <t>Completo (3 idiomas)</t>
         </is>
       </c>
-      <c r="H384" s="5" t="inlineStr"/>
+      <c r="H384" s="5" t="inlineStr">
+        <is>
+          <t>[EN: 'Connection' sounds more natural than 'meeting' in this context, and 'physical well-being' is more idiomatic than 'bodily well-being'.]</t>
+        </is>
+      </c>
     </row>
     <row r="385">
       <c r="A385" s="7" t="n">
@@ -14991,7 +15071,7 @@
       </c>
       <c r="E402" s="5" t="inlineStr">
         <is>
-          <t>Individual Session / Personal</t>
+          <t>Private Session / Personal</t>
         </is>
       </c>
       <c r="F402" s="5" t="inlineStr">
@@ -15004,7 +15084,11 @@
           <t>Completo (3 idiomas)</t>
         </is>
       </c>
-      <c r="H402" s="5" t="inlineStr"/>
+      <c r="H402" s="5" t="inlineStr">
+        <is>
+          <t>[EN: 'Private Session' is the standard English term for 1-on-1 classes, rather than 'Individual Session'.]</t>
+        </is>
+      </c>
     </row>
     <row r="403">
       <c r="A403" s="7" t="n">
@@ -15248,7 +15332,7 @@
       </c>
       <c r="F409" s="10" t="inlineStr">
         <is>
-          <t>Ta Kontakt</t>
+          <t>Ta kontakt</t>
         </is>
       </c>
       <c r="G409" s="11" t="inlineStr">
@@ -15256,7 +15340,11 @@
           <t>Completo (3 idiomas)</t>
         </is>
       </c>
-      <c r="H409" s="10" t="inlineStr"/>
+      <c r="H409" s="10" t="inlineStr">
+        <is>
+          <t>[NO: In Norwegian, only the first word in a title or heading is capitalized, unless it's a proper noun.]</t>
+        </is>
+      </c>
     </row>
     <row r="410">
       <c r="A410" s="2" t="n">
@@ -15351,7 +15439,7 @@
       </c>
       <c r="E412" s="5" t="inlineStr">
         <is>
-          <t>Biostretch Corporate is designed for organizations that wish to create spaces of guided pause, active listening, and strengthening of physical and emotional well-being within the institutional environment. Especially recommended for:</t>
+          <t>Biostretch Corporate is designed for organizations that wish to create spaces for guided pauses, active listening, and strengthening physical and emotional well-being within the corporate environment. Especially recommended for:</t>
         </is>
       </c>
       <c r="F412" s="5" t="inlineStr">
@@ -15364,7 +15452,11 @@
           <t>Completo (3 idiomas)</t>
         </is>
       </c>
-      <c r="H412" s="5" t="inlineStr"/>
+      <c r="H412" s="5" t="inlineStr">
+        <is>
+          <t>[EN: Changed 'spaces of guided pause' to 'spaces for guided pauses' and 'institutional' to 'corporate' for better flow and natural business English.]</t>
+        </is>
+      </c>
     </row>
     <row r="413">
       <c r="A413" s="7" t="n">
@@ -16724,7 +16816,7 @@
       </c>
       <c r="F450" s="5" t="inlineStr">
         <is>
-          <t>Fysiologi og Bevissthet</t>
+          <t>Fysiologi og bevissthet</t>
         </is>
       </c>
       <c r="G450" s="6" t="inlineStr">
@@ -16732,7 +16824,11 @@
           <t>Completo (3 idiomas)</t>
         </is>
       </c>
-      <c r="H450" s="5" t="inlineStr"/>
+      <c r="H450" s="5" t="inlineStr">
+        <is>
+          <t>[NO: In Norwegian, only the first word in a heading is capitalized.]</t>
+        </is>
+      </c>
     </row>
     <row r="451">
       <c r="A451" s="7" t="n">
@@ -17120,7 +17216,7 @@
       </c>
       <c r="F461" s="10" t="inlineStr">
         <is>
-          <t>Tilsteværelse og Bærekraft</t>
+          <t>Tilstedeværelse og bærekraft</t>
         </is>
       </c>
       <c r="G461" s="11" t="inlineStr">
@@ -17128,7 +17224,11 @@
           <t>Completo (3 idiomas)</t>
         </is>
       </c>
-      <c r="H461" s="10" t="inlineStr"/>
+      <c r="H461" s="10" t="inlineStr">
+        <is>
+          <t>[NO: Fixed typo 'Tilsteværelse' to 'Tilstedeværelse' and used correct Norwegian capitalization.]</t>
+        </is>
+      </c>
     </row>
     <row r="462">
       <c r="A462" s="2" t="n">
@@ -17367,7 +17467,7 @@
       </c>
       <c r="E468" s="5" t="inlineStr">
         <is>
-          <t>Foster healthier, more sustainable, and deeply humane workplace relations.</t>
+          <t>Build healthier, more sustainable, and deeply human workplace relationships.</t>
         </is>
       </c>
       <c r="F468" s="5" t="inlineStr">
@@ -17380,7 +17480,11 @@
           <t>Completo (3 idiomas)</t>
         </is>
       </c>
-      <c r="H468" s="5" t="inlineStr"/>
+      <c r="H468" s="5" t="inlineStr">
+        <is>
+          <t>[EN: 'Human' or 'human-centered' is more appropriate than 'humane' in a corporate relationship context. 'Relationships' is more common than 'relations' here.]</t>
+        </is>
+      </c>
     </row>
     <row r="469">
       <c r="A469" s="7" t="n">
@@ -17516,7 +17620,7 @@
       </c>
       <c r="F472" s="5" t="inlineStr">
         <is>
-          <t>Egenomsorg og Arbeidsmiljø</t>
+          <t>Egenomsorg og arbeidsmiljø</t>
         </is>
       </c>
       <c r="G472" s="6" t="inlineStr">
@@ -17524,7 +17628,11 @@
           <t>Completo (3 idiomas)</t>
         </is>
       </c>
-      <c r="H472" s="5" t="inlineStr"/>
+      <c r="H472" s="5" t="inlineStr">
+        <is>
+          <t>[NO: Corrected capitalization for Norwegian.]</t>
+        </is>
+      </c>
     </row>
     <row r="473">
       <c r="A473" s="7" t="n">
@@ -17547,7 +17655,7 @@
       </c>
       <c r="E473" s="10" t="inlineStr">
         <is>
-          <t>Through practices that combine movement, stretching, breathing, and attention to the body, employees are invited to step out of automatic mode and develop a more conscious relationship with their posture, movements, and well-being.</t>
+          <t>Through practices that combine movement, stretching, breathwork, and body awareness, employees are invited to step out of autopilot and develop a more conscious relationship with their posture, movements, and overall well-being.</t>
         </is>
       </c>
       <c r="F473" s="10" t="inlineStr">
@@ -17560,7 +17668,11 @@
           <t>Completo (3 idiomas)</t>
         </is>
       </c>
-      <c r="H473" s="10" t="inlineStr"/>
+      <c r="H473" s="10" t="inlineStr">
+        <is>
+          <t>[EN: 'Autopilot' is more idiomatic than 'automatic mode', and 'breathwork' and 'body awareness' sound more natural for wellness copy.]</t>
+        </is>
+      </c>
     </row>
     <row r="474">
       <c r="A474" s="2" t="n">
@@ -17583,12 +17695,12 @@
       </c>
       <c r="E474" s="5" t="inlineStr">
         <is>
-          <t>Every company has its own dynamics. Every team faces different physical and mental challenges throughout the workday. Long hours at the computer, repetitive tasks, many hours standing, pressure for results, and an intense routine can generate wear and accumulated tension that goes unnoticed, until the body sends its signals.</t>
+          <t>Every company has its own dynamics. Every team faces different physical and mental challenges throughout the workday. Long hours at the computer, repetitive tasks, many hours standing, pressure for results, and an intense routine can generate wear and tear, and accumulated tension that goes unnoticed—until the body sends its signals.</t>
         </is>
       </c>
       <c r="F474" s="5" t="inlineStr">
         <is>
-          <t>Hver bedrift har sin egen dynamikk. Hvert team møter ulike fysiske og mentale utfordringer gjennom arbeidsdagen. Lange perioder foran datamaskinen, repetitive oppgaver, mange timer stående, press for resultater og en intens rutine kan generere slitasje og oppsamlet spenning som går ubemerket hen, helt til kroppen gir sine signaler.</t>
+          <t>Hver bedrift har sin egen dynamikk. Hvert team møter ulike fysiske og mentale utfordringer gjennom arbeidsdagen. Lange perioder foran datamaskinen, repetitive oppgaver, mange timer stående, press for resultater og en intens rutine kan generere slitasje og oppsamlet spenning som går ubemerket hen, helt til kroppen sier ifra.</t>
         </is>
       </c>
       <c r="G474" s="6" t="inlineStr">
@@ -17596,7 +17708,11 @@
           <t>Completo (3 idiomas)</t>
         </is>
       </c>
-      <c r="H474" s="5" t="inlineStr"/>
+      <c r="H474" s="5" t="inlineStr">
+        <is>
+          <t>[EN: 'Wear and tear' is the standard English idiom for physical 'desgaste'. Added an em-dash for a slightly more poetic rhythm.] | [NO: 'sier ifra' is a much more natural and idiomatic Norwegian expression for 'gives its signals'.]</t>
+        </is>
+      </c>
     </row>
     <row r="475">
       <c r="A475" s="7" t="n">
@@ -17619,7 +17735,7 @@
       </c>
       <c r="E475" s="10" t="inlineStr">
         <is>
-          <t>That is why Biostretch is always adapted to the characteristics and needs of each organization. The practices are built to offer an inclusive and meaningful experience, respecting different ages, profiles, and fitness levels. It is not workplace gymnastics. It is consciousness in movement.</t>
+          <t>That is why Biostretch is always adapted to the characteristics and needs of each organization. The practices are built to offer an inclusive and meaningful experience, respecting different ages, profiles, and fitness levels. It is not just workplace stretching. It is consciousness in movement.</t>
         </is>
       </c>
       <c r="F475" s="10" t="inlineStr">
@@ -17632,7 +17748,11 @@
           <t>Completo (3 idiomas)</t>
         </is>
       </c>
-      <c r="H475" s="10" t="inlineStr"/>
+      <c r="H475" s="10" t="inlineStr">
+        <is>
+          <t>[EN: 'Workplace gymnastics' sounds unnatural in English; 'workplace stretching' correctly conveys 'ginástica laboral'.]</t>
+        </is>
+      </c>
     </row>
     <row r="476">
       <c r="A476" s="2" t="n">
@@ -18123,7 +18243,7 @@
       </c>
       <c r="E489" s="10" t="inlineStr">
         <is>
-          <t>Dance entered my life through medical advice. At seven, classical ballet was recommended to align my foot posture. The initial obligation became a fascination. The discipline of the barres and the enthusiasm of master João Luiz Rolla marked the beginning of a journey guided by movement.</t>
+          <t>Dance entered my life through medical advice. At seven, classical ballet was recommended to correct my foot posture. The initial obligation soon became a fascination. The discipline of the barre and the enthusiasm of master João Luiz Rolla marked the beginning of a journey guided by movement.</t>
         </is>
       </c>
       <c r="F489" s="10" t="inlineStr">
@@ -18136,7 +18256,11 @@
           <t>Completo (3 idiomas)</t>
         </is>
       </c>
-      <c r="H489" s="10" t="inlineStr"/>
+      <c r="H489" s="10" t="inlineStr">
+        <is>
+          <t>[EN: 'Correct my foot posture' is more accurate to 'corrigir', and 'the barre' is the standard singular term used in ballet contexts rather than 'barres'.]</t>
+        </is>
+      </c>
     </row>
     <row r="490">
       <c r="A490" s="2" t="n">
@@ -18632,7 +18756,7 @@
       </c>
       <c r="F503" s="10" t="inlineStr">
         <is>
-          <t>Utforsk Workshops</t>
+          <t>Utforsk workshops</t>
         </is>
       </c>
       <c r="G503" s="11" t="inlineStr">
@@ -18640,7 +18764,11 @@
           <t>Completo (3 idiomas)</t>
         </is>
       </c>
-      <c r="H503" s="10" t="inlineStr"/>
+      <c r="H503" s="10" t="inlineStr">
+        <is>
+          <t>[NO: Capitalization rules in Norwegian.]</t>
+        </is>
+      </c>
     </row>
     <row r="504">
       <c r="A504" s="2" t="n">
@@ -18776,7 +18904,7 @@
       </c>
       <c r="F507" s="10" t="inlineStr">
         <is>
-          <t>er en sosial organisasjon som ble født for å bygge disse stedene. Rom hvor dans ikke bare er opptreden, men fremfor alt er tilstedeværelse. Hvor bevegelse er mer enn trening eller tøying, det er lytting og uttrykk. Hvor kunst ikke er et mål, men begynnelsen på et møte.</t>
+          <t>er en sosial organisasjon som ble skapt for å bygge disse stedene. Rom hvor dans ikke bare er opptreden, men fremfor alt er tilstedeværelse. Hvor bevegelse er mer enn trening eller tøying, det er lytting og uttrykk. Hvor kunst ikke er et mål, men begynnelsen på et møte.</t>
         </is>
       </c>
       <c r="G507" s="11" t="inlineStr">
@@ -18784,7 +18912,11 @@
           <t>Completo (3 idiomas)</t>
         </is>
       </c>
-      <c r="H507" s="10" t="inlineStr"/>
+      <c r="H507" s="10" t="inlineStr">
+        <is>
+          <t>[NO: 'ble født' (was born) is too literal for an organization in Norwegian. 'ble skapt' (was created) or 'ble til' sounds much more natural.]</t>
+        </is>
+      </c>
     </row>
     <row r="508">
       <c r="A508" s="2" t="n">
@@ -20751,7 +20883,7 @@
       </c>
       <c r="E562" s="5" t="inlineStr">
         <is>
-          <t>&lt;p&gt;The methodologies taught (Biostretch and Be The Dance) are practices focused on movement, breathing, and body awareness. &lt;strong&gt;They do not replace medical, physiotherapeutic, or psychological diagnoses or treatments.&lt;/strong&gt; You assume the responsibility to respect your body's limits and seek medical clearance if you have pre-existing conditions.&lt;/p&gt;</t>
+          <t>&lt;p&gt;The methodologies taught (Biostretch and Be The Dance) are practices focused on movement, breathing, and body awareness. &lt;strong&gt;They do not replace medical, physical therapy, or psychological diagnoses or treatments.&lt;/strong&gt; You assume the responsibility to respect your body's limits and seek medical clearance if you have pre-existing conditions.&lt;/p&gt;</t>
         </is>
       </c>
       <c r="F562" s="5" t="inlineStr">
@@ -20764,7 +20896,11 @@
           <t>Completo (3 idiomas)</t>
         </is>
       </c>
-      <c r="H562" s="5" t="inlineStr"/>
+      <c r="H562" s="5" t="inlineStr">
+        <is>
+          <t>[EN: 'Physical therapy' is the much more common and natural term in English compared to 'physiotherapeutic'.]</t>
+        </is>
+      </c>
     </row>
     <row r="563">
       <c r="A563" s="7" t="n">
@@ -21440,7 +21576,7 @@
       </c>
       <c r="F581" s="10" t="inlineStr">
         <is>
-          <t>Sosialt Prosjekt</t>
+          <t>Sosialt prosjekt</t>
         </is>
       </c>
       <c r="G581" s="11" t="inlineStr">
@@ -21448,7 +21584,11 @@
           <t>Completo (3 idiomas)</t>
         </is>
       </c>
-      <c r="H581" s="10" t="inlineStr"/>
+      <c r="H581" s="10" t="inlineStr">
+        <is>
+          <t>[NO: Corrected capitalization for Norwegian.]</t>
+        </is>
+      </c>
     </row>
     <row r="582">
       <c r="A582" s="2" t="n">
@@ -21759,12 +21899,12 @@
       </c>
       <c r="E590" s="5" t="inlineStr">
         <is>
-          <t>Filosofia e conceito do Be the Dance...</t>
+          <t>Philosophy and concept of Be the Dance...</t>
         </is>
       </c>
       <c r="F590" s="5" t="inlineStr">
         <is>
-          <t>Filosofia e conceito do Be the Dance...</t>
+          <t>Filosofi og konsept bak Be the Dance...</t>
         </is>
       </c>
       <c r="G590" s="6" t="inlineStr">
@@ -21772,7 +21912,11 @@
           <t>Completo (3 idiomas)</t>
         </is>
       </c>
-      <c r="H590" s="5" t="inlineStr"/>
+      <c r="H590" s="5" t="inlineStr">
+        <is>
+          <t>[EN: The text was left in Portuguese and needed translation.] | [NO: Oversatt fra portugisisk med naturlig ordlyd.]</t>
+        </is>
+      </c>
     </row>
     <row r="591">
       <c r="A591" s="7" t="n">
@@ -22155,12 +22299,12 @@
       </c>
       <c r="E601" s="10" t="inlineStr">
         <is>
-          <t>Because I believe dance is not a privilege of those born flexible, those who started at age four, or those who learned to count eight beats. Dance is in our genes. It is in the impulse to sway when we hear music. In the body that moves when we are happy. In the spontaneous gesture. In the breath. In the rhythm. In the desire to celebrate, seduce, play, and be free. Perhaps we all have the dance inside us and it just needs a stimulus to appear.</t>
+          <t>Because I believe dance is not a privilege of those born flexible, those who started at age four, or those who learned to count in eights. Dance is in our genes. It is in the impulse to sway when we hear music. In the body that moves when we are happy. In the spontaneous gesture. In the breath. In the rhythm. In the desire to celebrate, to seduce, to play, and to be free. Perhaps we all have the dance inside us and it just needs a spark to emerge.</t>
         </is>
       </c>
       <c r="F601" s="10" t="inlineStr">
         <is>
-          <t>For jeg tror at dans ikke er et privilegium for dem som er født fleksible, dem som begynte som fireåringer, eller dem som lærte å telle åtte slag. Dansen ligger i genene våre. Den ligger i impulsen til å gynge når vi hører musikk. I kroppen som beveger seg når vi er glade. I den spontane gesten. I pusten. I rytmen. I ønsket om å feire, forføre, leke og frigjøre seg. Kanskje vi alle har dansen inni oss, og det trengs bare et stimuli for å la den komme frem.</t>
+          <t>For jeg tror at dans ikke er et privilegium for dem som er født fleksible, dem som begynte som fireåringer, eller dem som lærte å telle åtte slag. Dansen ligger i genene våre. Den ligger i impulsen til å gynge når vi hører musikk. I kroppen som beveger seg når vi er glade. I den spontane gesten. I pusten. I rytmen. I ønsket om å feire, forføre, leke og frigjøre seg. Kanskje vi alle har dansen inni oss, og at det bare trengs en stimulans for å la den komme frem.</t>
         </is>
       </c>
       <c r="G601" s="11" t="inlineStr">
@@ -22168,7 +22312,11 @@
           <t>Completo (3 idiomas)</t>
         </is>
       </c>
-      <c r="H601" s="10" t="inlineStr"/>
+      <c r="H601" s="10" t="inlineStr">
+        <is>
+          <t>[EN: 'Count in eights' is standard dance terminology. 'Spark to emerge' feels slightly more poetic and natural than 'stimulus to appear'.] | [NO: 'et stimuli' is grammatically incorrect in Norwegian (should be 'et stimulus' or 'en stimulans'). 'en stimulans' fits well here.]</t>
+        </is>
+      </c>
     </row>
     <row r="602">
       <c r="A602" s="2" t="n">
@@ -22227,7 +22375,7 @@
       </c>
       <c r="E603" s="10" t="inlineStr">
         <is>
-          <t>[SILVER]I started to see the body as a passage.</t>
+          <t>[SILVER]I began to see the body as a vessel.</t>
         </is>
       </c>
       <c r="F603" s="10" t="inlineStr">
@@ -22240,7 +22388,11 @@
           <t>Completo (3 idiomas)</t>
         </is>
       </c>
-      <c r="H603" s="10" t="inlineStr"/>
+      <c r="H603" s="10" t="inlineStr">
+        <is>
+          <t>[EN: 'Vessel' or 'conduit' sounds more natural and poetic in this context than the literal 'passage'.]</t>
+        </is>
+      </c>
     </row>
     <row r="604">
       <c r="A604" s="2" t="n">
@@ -22299,7 +22451,7 @@
       </c>
       <c r="E605" s="10" t="inlineStr">
         <is>
-          <t>A place of listening. A territory of discovery. An instrument through which we can cross our own borders and find a form of expression that is unique, personal, and genuine. That is how Be The Dance began to take shape.</t>
+          <t>A place of listening. A landscape of discovery. An instrument through which we can push past our own boundaries and find a form of expression that is unique, personal, and genuine. That is how Be The Dance began to take shape.</t>
         </is>
       </c>
       <c r="F605" s="10" t="inlineStr">
@@ -22312,7 +22464,11 @@
           <t>Completo (3 idiomas)</t>
         </is>
       </c>
-      <c r="H605" s="10" t="inlineStr"/>
+      <c r="H605" s="10" t="inlineStr">
+        <is>
+          <t>[EN: 'Landscape of discovery' and 'push past our own boundaries' sound more natural and poetic.]</t>
+        </is>
+      </c>
     </row>
     <row r="606">
       <c r="A606" s="2" t="n">
@@ -22335,12 +22491,12 @@
       </c>
       <c r="E606" s="5" t="inlineStr">
         <is>
-          <t>But I soon realized that this investigation could also be profoundly transformative for professional dancers. Because I know this path from the inside. I know how much a dancer can dedicate years to perfecting technique. The correct position. The highest jump. The perfect line. Absolute control of the body.</t>
+          <t>But I soon realized that this investigation could also be profoundly transformative for professional dancers. Because I know this journey intimately. I know how a dancer can dedicate years to perfecting their technique. The correct position. The highest jump. The perfect line. Absolute control of the body.</t>
         </is>
       </c>
       <c r="F606" s="5" t="inlineStr">
         <is>
-          <t>Men jeg innså snart at denne utforskningen også kunne være dypt transformerende for profesjonelle dansere. For jeg kjenner denne veien fra innsiden. Jeg vet hvor mye en danser kan dedikere av år for å perfeksjonere teknikken. Den riktige posisjonen. Det høyeste hoppet. Den perfekte linjen. Den absolutte kontrollen over kroppen.</t>
+          <t>Men jeg innså snart at denne utforskningen også kunne være dypt transformerende for profesjonelle dansere. For jeg kjenner denne veien fra innsiden. Jeg vet hvor mange år en danser kan vie til å perfeksjonere teknikken. Den riktige posisjonen. Det høyeste hoppet. Den perfekte linjen. Den absolutte kontrollen over kroppen.</t>
         </is>
       </c>
       <c r="G606" s="6" t="inlineStr">
@@ -22348,7 +22504,11 @@
           <t>Completo (3 idiomas)</t>
         </is>
       </c>
-      <c r="H606" s="5" t="inlineStr"/>
+      <c r="H606" s="5" t="inlineStr">
+        <is>
+          <t>[EN: 'Journey intimately' and 'how a dancer can dedicate years' flows much better in native English.] | [NO: Phrasing: 'dedikere av år for å' is unidiomatic. 'vie til' or 'bruke årevis på' sounds much more native.]</t>
+        </is>
+      </c>
     </row>
     <row r="607">
       <c r="A607" s="7" t="n">
@@ -22479,7 +22639,7 @@
       </c>
       <c r="E610" s="5" t="inlineStr">
         <is>
-          <t>Because maybe you don't need to know. Maybe you just need to start. And then discover that the dance was already there. Waiting for you.</t>
+          <t>Because maybe you don't need to know how. Maybe you just need to start. And then discover that the dance was already there. Waiting for you.</t>
         </is>
       </c>
       <c r="F610" s="5" t="inlineStr">
@@ -22492,7 +22652,11 @@
           <t>Completo (3 idiomas)</t>
         </is>
       </c>
-      <c r="H610" s="5" t="inlineStr"/>
+      <c r="H610" s="5" t="inlineStr">
+        <is>
+          <t>[EN: In English, 'know how' completes the thought regarding the previous sentence about 'not knowing how to dance'.]</t>
+        </is>
+      </c>
     </row>
     <row r="611">
       <c r="A611" s="7" t="n">
@@ -22842,7 +23006,7 @@
       </c>
       <c r="E620" s="5" t="inlineStr">
         <is>
-          <t>People who might never have imagined doing so in public were there, moving their bodies, meeting others, laughing, playing, experimenting. Dance left the stage. And found life.</t>
+          <t>People who might never have imagined doing so in public were there, moving their bodies, meeting others, laughing, playing, experimenting. Dance stepped off the stage and came alive.</t>
         </is>
       </c>
       <c r="F620" s="5" t="inlineStr">
@@ -22855,7 +23019,11 @@
           <t>Completo (3 idiomas)</t>
         </is>
       </c>
-      <c r="H620" s="5" t="inlineStr"/>
+      <c r="H620" s="5" t="inlineStr">
+        <is>
+          <t>[EN: 'Stepped off the stage and came alive' is much more idiomatic and poetic.]</t>
+        </is>
+      </c>
     </row>
     <row r="621">
       <c r="A621" s="7" t="n">
@@ -22986,12 +23154,12 @@
       </c>
       <c r="E624" s="5" t="inlineStr">
         <is>
-          <t>é um programa de quatro workshops de dança.</t>
+          <t>is a program consisting of four dance workshops.</t>
         </is>
       </c>
       <c r="F624" s="5" t="inlineStr">
         <is>
-          <t>é um programa de quatro workshops de dança.</t>
+          <t>er et program bestående av fire danseworkshops.</t>
         </is>
       </c>
       <c r="G624" s="6" t="inlineStr">
@@ -22999,7 +23167,11 @@
           <t>Completo (3 idiomas)</t>
         </is>
       </c>
-      <c r="H624" s="5" t="inlineStr"/>
+      <c r="H624" s="5" t="inlineStr">
+        <is>
+          <t>[EN: Translation was missing.] | [NO: Was not translated.]</t>
+        </is>
+      </c>
     </row>
     <row r="625">
       <c r="A625" s="7" t="n">
@@ -23022,12 +23194,12 @@
       </c>
       <c r="E625" s="10" t="inlineStr">
         <is>
-          <t>Foi desenhado para você explorar o movimento como caminho de presença, expressão e autoconhecimento, despertando algo essencial e único que já existe em você: sua própria dança.</t>
+          <t>It was designed for you to explore movement as a path to presence, expression, and self-discovery, awakening something essential and unique that already exists within you: your very own dance.</t>
         </is>
       </c>
       <c r="F625" s="10" t="inlineStr">
         <is>
-          <t>Foi desenhado para você explorar o movimento como caminho de presença, expressão e autoconhecimento, despertando algo essencial e único que já existe em você: sua própria dança.</t>
+          <t>Det er designet for at du skal kunne utforske bevegelse som en vei til tilstedeværelse, uttrykk og selvinnsikt, og vekke noe essensielt og unikt som allerede finnes i deg: din egen dans.</t>
         </is>
       </c>
       <c r="G625" s="11" t="inlineStr">
@@ -23035,7 +23207,11 @@
           <t>Completo (3 idiomas)</t>
         </is>
       </c>
-      <c r="H625" s="10" t="inlineStr"/>
+      <c r="H625" s="10" t="inlineStr">
+        <is>
+          <t>[EN: Translation was missing.] | [NO: Was not translated.]</t>
+        </is>
+      </c>
     </row>
     <row r="626">
       <c r="A626" s="2" t="n">
@@ -23094,12 +23270,12 @@
       </c>
       <c r="E627" s="10" t="inlineStr">
         <is>
-          <t>A dança pode nascer no corpo de qualquer pessoa que se permita mover.</t>
+          <t>Dance can be born in the body of anyone who allows themselves to move.</t>
         </is>
       </c>
       <c r="F627" s="10" t="inlineStr">
         <is>
-          <t>A dança pode nascer no corpo de qualquer pessoa que se permita mover.</t>
+          <t>Dans kan oppstå i kroppen til enhver person som tillater seg å bevege seg.</t>
         </is>
       </c>
       <c r="G627" s="11" t="inlineStr">
@@ -23107,7 +23283,11 @@
           <t>Completo (3 idiomas)</t>
         </is>
       </c>
-      <c r="H627" s="10" t="inlineStr"/>
+      <c r="H627" s="10" t="inlineStr">
+        <is>
+          <t>[EN: Translation was missing.] | [NO: Was not translated.]</t>
+        </is>
+      </c>
     </row>
     <row r="628">
       <c r="A628" s="2" t="n">
@@ -23130,12 +23310,12 @@
       </c>
       <c r="E628" s="5" t="inlineStr">
         <is>
-          <t>Não há exigências.</t>
+          <t>There are no prerequisites.</t>
         </is>
       </c>
       <c r="F628" s="5" t="inlineStr">
         <is>
-          <t>Não há exigências.</t>
+          <t>Det stilles ingen krav.</t>
         </is>
       </c>
       <c r="G628" s="6" t="inlineStr">
@@ -23143,7 +23323,11 @@
           <t>Completo (3 idiomas)</t>
         </is>
       </c>
-      <c r="H628" s="5" t="inlineStr"/>
+      <c r="H628" s="5" t="inlineStr">
+        <is>
+          <t>[EN: Translation was missing.] | [NO: Was not translated.]</t>
+        </is>
+      </c>
     </row>
     <row r="629">
       <c r="A629" s="7" t="n">
@@ -23166,12 +23350,12 @@
       </c>
       <c r="E629" s="10" t="inlineStr">
         <is>
-          <t>Basta sentir e permitir que o movimento se expresse.</t>
+          <t>You just need to feel and allow the movement to express itself.</t>
         </is>
       </c>
       <c r="F629" s="10" t="inlineStr">
         <is>
-          <t>Basta sentir e permitir que o movimento se expresse.</t>
+          <t>Det handler bare om å føle og la bevegelsen uttrykke seg.</t>
         </is>
       </c>
       <c r="G629" s="11" t="inlineStr">
@@ -23179,7 +23363,11 @@
           <t>Completo (3 idiomas)</t>
         </is>
       </c>
-      <c r="H629" s="10" t="inlineStr"/>
+      <c r="H629" s="10" t="inlineStr">
+        <is>
+          <t>[EN: Translation was missing.] | [NO: Was not translated.]</t>
+        </is>
+      </c>
     </row>
     <row r="630">
       <c r="A630" s="2" t="n">
@@ -23202,12 +23390,12 @@
       </c>
       <c r="E630" s="5" t="inlineStr">
         <is>
-          <t>Em qualquer idade ou condição física, é possível descobrir uma forma própria de dançar.</t>
+          <t>At any age or physical condition, it is possible to discover your own way of dancing.</t>
         </is>
       </c>
       <c r="F630" s="5" t="inlineStr">
         <is>
-          <t>Em qualquer idade ou condição física, é possível descobrir uma forma própria de dançar.</t>
+          <t>Uansett alder eller fysisk form er det mulig å oppdage sin egen måte å danse på.</t>
         </is>
       </c>
       <c r="G630" s="6" t="inlineStr">
@@ -23215,7 +23403,11 @@
           <t>Completo (3 idiomas)</t>
         </is>
       </c>
-      <c r="H630" s="5" t="inlineStr"/>
+      <c r="H630" s="5" t="inlineStr">
+        <is>
+          <t>[EN: Translation was missing.] | [NO: Was not translated.]</t>
+        </is>
+      </c>
     </row>
     <row r="631">
       <c r="A631" s="7" t="n">
@@ -23238,12 +23430,12 @@
       </c>
       <c r="E631" s="10" t="inlineStr">
         <is>
-          <t>BE THE DANCE É PARA TODOS</t>
+          <t>BE THE DANCE IS FOR EVERYONE</t>
         </is>
       </c>
       <c r="F631" s="10" t="inlineStr">
         <is>
-          <t>BE THE DANCE É PARA TODOS</t>
+          <t>BE THE DANCE ER FOR ALLE</t>
         </is>
       </c>
       <c r="G631" s="11" t="inlineStr">
@@ -23251,7 +23443,11 @@
           <t>Completo (3 idiomas)</t>
         </is>
       </c>
-      <c r="H631" s="10" t="inlineStr"/>
+      <c r="H631" s="10" t="inlineStr">
+        <is>
+          <t>[EN: Translation was missing.] | [NO: Was not translated.]</t>
+        </is>
+      </c>
     </row>
     <row r="632">
       <c r="A632" s="2" t="n">
@@ -23274,12 +23470,12 @@
       </c>
       <c r="E632" s="5" t="inlineStr">
         <is>
-          <t>Não está restrita a uma técnica, a um estilo pré-definido ou a um talento especial.</t>
+          <t>It is not restricted to a technique, a predefined style, or a special talent.</t>
         </is>
       </c>
       <c r="F632" s="5" t="inlineStr">
         <is>
-          <t>Não está restrita a uma técnica, a um estilo pré-definido ou a um talento especial.</t>
+          <t>Den er ikke begrenset til en bestemt teknikk, en forhåndsdefinert stil eller et spesielt talent.</t>
         </is>
       </c>
       <c r="G632" s="6" t="inlineStr">
@@ -23287,7 +23483,11 @@
           <t>Completo (3 idiomas)</t>
         </is>
       </c>
-      <c r="H632" s="5" t="inlineStr"/>
+      <c r="H632" s="5" t="inlineStr">
+        <is>
+          <t>[EN: Translation was missing.] | [NO: Was not translated.]</t>
+        </is>
+      </c>
     </row>
     <row r="633">
       <c r="A633" s="7" t="n">
@@ -23310,12 +23510,12 @@
       </c>
       <c r="E633" s="10" t="inlineStr">
         <is>
-          <t>Ela existe em cada pessoa, como uma criatividade inerente pronta para ganhar forma por meio do corpo.</t>
+          <t>It exists in everyone, as an inherent creativity ready to take shape through the body.</t>
         </is>
       </c>
       <c r="F633" s="10" t="inlineStr">
         <is>
-          <t>Ela existe em cada pessoa, como uma criatividade inerente pronta para ganhar forma por meio do corpo.</t>
+          <t>Den finnes i hver og en av oss, som en iboende kreativitet klar til å ta form gjennom kroppen.</t>
         </is>
       </c>
       <c r="G633" s="11" t="inlineStr">
@@ -23323,7 +23523,11 @@
           <t>Completo (3 idiomas)</t>
         </is>
       </c>
-      <c r="H633" s="10" t="inlineStr"/>
+      <c r="H633" s="10" t="inlineStr">
+        <is>
+          <t>[EN: Translation was missing.] | [NO: Was not translated.]</t>
+        </is>
+      </c>
     </row>
     <row r="634">
       <c r="A634" s="2" t="n">
@@ -23346,12 +23550,12 @@
       </c>
       <c r="E634" s="5" t="inlineStr">
         <is>
-          <t>ONDE ESTÁ A DANÇA?</t>
+          <t>WHERE IS THE DANCE?</t>
         </is>
       </c>
       <c r="F634" s="5" t="inlineStr">
         <is>
-          <t>ONDE ESTÁ A DANÇA?</t>
+          <t>HVOR ER DANSEN?</t>
         </is>
       </c>
       <c r="G634" s="6" t="inlineStr">
@@ -23359,7 +23563,11 @@
           <t>Completo (3 idiomas)</t>
         </is>
       </c>
-      <c r="H634" s="5" t="inlineStr"/>
+      <c r="H634" s="5" t="inlineStr">
+        <is>
+          <t>[EN: Translation was missing.] | [NO: Was not translated.]</t>
+        </is>
+      </c>
     </row>
     <row r="635">
       <c r="A635" s="7" t="n">
@@ -23382,12 +23590,12 @@
       </c>
       <c r="E635" s="10" t="inlineStr">
         <is>
-          <t>A dança nos acompanha há milênios, como ritual, celebração e expressão artística. Ainda que você não lembre, há no corpo uma memória de movimento, uma capacidade de sentir, criar e dançar.</t>
+          <t>Dance has accompanied us for millennia, as ritual, celebration, and artistic expression. Even if you don't remember, there is a memory of movement in the body, an ability to feel, create, and dance.</t>
         </is>
       </c>
       <c r="F635" s="10" t="inlineStr">
         <is>
-          <t>A dança nos acompanha há milênios, como ritual, celebração e expressão artística. Ainda que você não lembre, há no corpo uma memória de movimento, uma capacidade de sentir, criar e dançar.</t>
+          <t>Dansen har fulgt oss i årtusener, som ritual, feiring og kunstnerisk uttrykk. Selv om du kanskje ikke husker det, bærer kroppen på et bevegelsesminne, en evne til å føle, skape og danse.</t>
         </is>
       </c>
       <c r="G635" s="11" t="inlineStr">
@@ -23395,7 +23603,11 @@
           <t>Completo (3 idiomas)</t>
         </is>
       </c>
-      <c r="H635" s="10" t="inlineStr"/>
+      <c r="H635" s="10" t="inlineStr">
+        <is>
+          <t>[EN: Translation was missing.] | [NO: Was not translated.]</t>
+        </is>
+      </c>
     </row>
     <row r="636">
       <c r="A636" s="2" t="n">
@@ -23418,12 +23630,12 @@
       </c>
       <c r="E636" s="5" t="inlineStr">
         <is>
-          <t>Ao criar um diálogo sensível entre música e corpo, abrimos a possibilidade de explorar novos caminhos de movimento. Ir além do conhecido permite que novas formas de expressão possam emergir.</t>
+          <t>By creating a sensitive dialogue between music and body, we open up the possibility of exploring new paths of movement. Going beyond the known allows new forms of expression to emerge.</t>
         </is>
       </c>
       <c r="F636" s="5" t="inlineStr">
         <is>
-          <t>Ao criar um diálogo sensível entre música e corpo, abrimos a possibilidade de explorar novos caminhos de movimento. Ir além do conhecido permite que novas formas de expressão possam emergir.</t>
+          <t>Ved å skape en sensitiv dialog mellom musikk og kropp, åpner vi muligheten for å utforske nye bevegelsesveier. Å gå utover det kjente lar nye uttrykksformer vokse frem.</t>
         </is>
       </c>
       <c r="G636" s="6" t="inlineStr">
@@ -23431,7 +23643,11 @@
           <t>Completo (3 idiomas)</t>
         </is>
       </c>
-      <c r="H636" s="5" t="inlineStr"/>
+      <c r="H636" s="5" t="inlineStr">
+        <is>
+          <t>[EN: Translation was missing.] | [NO: Was not translated.]</t>
+        </is>
+      </c>
     </row>
     <row r="637">
       <c r="A637" s="7" t="n">
@@ -23454,12 +23670,12 @@
       </c>
       <c r="E637" s="10" t="inlineStr">
         <is>
-          <t>A dança acontece para além do controle e da busca por uma forma ideal. Quando nos permitimos estar presentes, uma expressão mais autêntica e única pode emergir do corpo.</t>
+          <t>Dance happens beyond control and the search for an ideal form. When we allow ourselves to be present, a more authentic and unique expression can emerge from the body.</t>
         </is>
       </c>
       <c r="F637" s="10" t="inlineStr">
         <is>
-          <t>A dança acontece para além do controle e da busca por uma forma ideal. Quando nos permitimos estar presentes, uma expressão mais autêntica e única pode emergir do corpo.</t>
+          <t>Dansen skjer forbi kontroll og jakten på en ideell form. Når vi tillater oss å være til stede, kan et mer autentisk og unikt uttrykk vokse frem fra kroppen.</t>
         </is>
       </c>
       <c r="G637" s="11" t="inlineStr">
@@ -23467,7 +23683,11 @@
           <t>Completo (3 idiomas)</t>
         </is>
       </c>
-      <c r="H637" s="10" t="inlineStr"/>
+      <c r="H637" s="10" t="inlineStr">
+        <is>
+          <t>[EN: Translation was missing.] | [NO: Was not translated.]</t>
+        </is>
+      </c>
     </row>
     <row r="638">
       <c r="A638" s="2" t="n">
@@ -23490,12 +23710,12 @@
       </c>
       <c r="E638" s="5" t="inlineStr">
         <is>
-          <t>COMO ACONTECE A DANÇA?</t>
+          <t>HOW DOES DANCE HAPPEN?</t>
         </is>
       </c>
       <c r="F638" s="5" t="inlineStr">
         <is>
-          <t>COMO ACONTECE A DANÇA?</t>
+          <t>HVORDAN SKJER DANSEN?</t>
         </is>
       </c>
       <c r="G638" s="6" t="inlineStr">
@@ -23503,7 +23723,11 @@
           <t>Completo (3 idiomas)</t>
         </is>
       </c>
-      <c r="H638" s="5" t="inlineStr"/>
+      <c r="H638" s="5" t="inlineStr">
+        <is>
+          <t>[EN: Translation was missing.] | [NO: Was not translated.]</t>
+        </is>
+      </c>
     </row>
     <row r="639">
       <c r="A639" s="7" t="n">
@@ -23526,12 +23750,12 @@
       </c>
       <c r="E639" s="10" t="inlineStr">
         <is>
-          <t>• Favorecer o relaxamento profundo e contribuir para a redução do estresse.</t>
+          <t>• Promotes deep relaxation and contributes to stress reduction.</t>
         </is>
       </c>
       <c r="F639" s="10" t="inlineStr">
         <is>
-          <t>• Favorecer o relaxamento profundo e contribuir para a redução do estresse.</t>
+          <t>• Fremme dyp avspenning og bidra til å redusere stress.</t>
         </is>
       </c>
       <c r="G639" s="11" t="inlineStr">
@@ -23539,7 +23763,11 @@
           <t>Completo (3 idiomas)</t>
         </is>
       </c>
-      <c r="H639" s="10" t="inlineStr"/>
+      <c r="H639" s="10" t="inlineStr">
+        <is>
+          <t>[EN: Translation was missing.] | [NO: Was not translated.]</t>
+        </is>
+      </c>
     </row>
     <row r="640">
       <c r="A640" s="2" t="n">
@@ -23562,12 +23790,12 @@
       </c>
       <c r="E640" s="5" t="inlineStr">
         <is>
-          <t>• Ampliar a energia, a disponibilidade corporal e a fluidez dos movimentos.</t>
+          <t>• Increases energy, physical readiness, and the fluidity of movements.</t>
         </is>
       </c>
       <c r="F640" s="5" t="inlineStr">
         <is>
-          <t>• Ampliar a energia, a disponibilidade corporal e a fluidez dos movimentos.</t>
+          <t>• Øke energien, kroppens tilgjengelighet og flyten i bevegelsene.</t>
         </is>
       </c>
       <c r="G640" s="6" t="inlineStr">
@@ -23575,7 +23803,11 @@
           <t>Completo (3 idiomas)</t>
         </is>
       </c>
-      <c r="H640" s="5" t="inlineStr"/>
+      <c r="H640" s="5" t="inlineStr">
+        <is>
+          <t>[EN: Translation was missing.] | [NO: Was not translated.]</t>
+        </is>
+      </c>
     </row>
     <row r="641">
       <c r="A641" s="7" t="n">
@@ -23598,12 +23830,12 @@
       </c>
       <c r="E641" s="10" t="inlineStr">
         <is>
-          <t>• Reconhecer movimentos naturais e ampliar a consciência corporal, criando espaço para uma expressão mais autêntica.</t>
+          <t>• Recognizes natural movements and expands body awareness, creating space for a more authentic expression.</t>
         </is>
       </c>
       <c r="F641" s="10" t="inlineStr">
         <is>
-          <t>• Reconhecer movimentos naturais e ampliar a consciência corporal, criando espaço para uma expressão mais autêntica.</t>
+          <t>• Gjenkjenne naturlige bevegelser og øke kroppsbevisstheten, og dermed skape rom for et mer autentisk uttrykk.</t>
         </is>
       </c>
       <c r="G641" s="11" t="inlineStr">
@@ -23611,7 +23843,11 @@
           <t>Completo (3 idiomas)</t>
         </is>
       </c>
-      <c r="H641" s="10" t="inlineStr"/>
+      <c r="H641" s="10" t="inlineStr">
+        <is>
+          <t>[EN: Translation was missing.] | [NO: Was not translated.]</t>
+        </is>
+      </c>
     </row>
     <row r="642">
       <c r="A642" s="2" t="n">
@@ -23634,12 +23870,12 @@
       </c>
       <c r="E642" s="5" t="inlineStr">
         <is>
-          <t>• Desenvolver a atenção, despertando os sentidos e aprofundando a presença.</t>
+          <t>• Develops attention, awakening the senses and deepening presence.</t>
         </is>
       </c>
       <c r="F642" s="5" t="inlineStr">
         <is>
-          <t>• Desenvolver a atenção, despertando os sentidos e aprofundando a presença.</t>
+          <t>• Utvikle oppmerksomheten, vekke sansene og utdype tilstedeværelsen.</t>
         </is>
       </c>
       <c r="G642" s="6" t="inlineStr">
@@ -23647,7 +23883,11 @@
           <t>Completo (3 idiomas)</t>
         </is>
       </c>
-      <c r="H642" s="5" t="inlineStr"/>
+      <c r="H642" s="5" t="inlineStr">
+        <is>
+          <t>[EN: Translation was missing.] | [NO: Was not translated.]</t>
+        </is>
+      </c>
     </row>
     <row r="643">
       <c r="A643" s="7" t="n">
@@ -23670,12 +23910,12 @@
       </c>
       <c r="E643" s="10" t="inlineStr">
         <is>
-          <t>• Explorar a relação entre respiração e movimento, descobrindo novas formas de dançar com mais liberdade.</t>
+          <t>• Explores the relationship between breath and movement, discovering new ways to dance with more freedom.</t>
         </is>
       </c>
       <c r="F643" s="10" t="inlineStr">
         <is>
-          <t>• Explorar a relação entre respiração e movimento, descobrindo novas formas de dançar com mais liberdade.</t>
+          <t>• Utforske forholdet mellom pust og bevegelse, og oppdage nye måter å danse på med større frihet.</t>
         </is>
       </c>
       <c r="G643" s="11" t="inlineStr">
@@ -23683,7 +23923,11 @@
           <t>Completo (3 idiomas)</t>
         </is>
       </c>
-      <c r="H643" s="10" t="inlineStr"/>
+      <c r="H643" s="10" t="inlineStr">
+        <is>
+          <t>[EN: Translation was missing.] | [NO: Was not translated.]</t>
+        </is>
+      </c>
     </row>
     <row r="644">
       <c r="A644" s="2" t="n">
@@ -23706,12 +23950,12 @@
       </c>
       <c r="E644" s="5" t="inlineStr">
         <is>
-          <t>• Ampliar a percepção reconhecendo as diferentes partes do corpo e as relações entre elas.</t>
+          <t>• Expands perception by recognizing the different parts of the body and the relationships between them.</t>
         </is>
       </c>
       <c r="F644" s="5" t="inlineStr">
         <is>
-          <t>• Ampliar a percepção reconhecendo as diferentes partes do corpo e as relações entre elas.</t>
+          <t>• Utvide persepsjonen ved å anerkjenne kroppens ulike deler og forholdet mellom dem.</t>
         </is>
       </c>
       <c r="G644" s="6" t="inlineStr">
@@ -23719,7 +23963,11 @@
           <t>Completo (3 idiomas)</t>
         </is>
       </c>
-      <c r="H644" s="5" t="inlineStr"/>
+      <c r="H644" s="5" t="inlineStr">
+        <is>
+          <t>[EN: Translation was missing.] | [NO: Was not translated.]</t>
+        </is>
+      </c>
     </row>
     <row r="645">
       <c r="A645" s="7" t="n">
@@ -23742,12 +23990,12 @@
       </c>
       <c r="E645" s="10" t="inlineStr">
         <is>
-          <t>QUAIS OS BENEFÍCIOS?</t>
+          <t>WHAT ARE THE BENEFITS?</t>
         </is>
       </c>
       <c r="F645" s="10" t="inlineStr">
         <is>
-          <t>QUAIS OS BENEFÍCIOS?</t>
+          <t>HVILKE ER FORDELENE?</t>
         </is>
       </c>
       <c r="G645" s="11" t="inlineStr">
@@ -23755,7 +24003,11 @@
           <t>Completo (3 idiomas)</t>
         </is>
       </c>
-      <c r="H645" s="10" t="inlineStr"/>
+      <c r="H645" s="10" t="inlineStr">
+        <is>
+          <t>[EN: Translation was missing.] | [NO: Was not translated.]</t>
+        </is>
+      </c>
     </row>
     <row r="646">
       <c r="A646" s="2" t="n">
@@ -23778,12 +24030,12 @@
       </c>
       <c r="E646" s="5" t="inlineStr">
         <is>
-          <t>Workshops que integram a consciência do movimento com práticas de dança e meditação, para você descobrir e expressar a dança que já existe em você.</t>
+          <t>Workshops that integrate movement awareness with dance and meditation practices, so you can discover and express the dance that already exists within you.</t>
         </is>
       </c>
       <c r="F646" s="5" t="inlineStr">
         <is>
-          <t>Workshops que integram a consciência do movimento com práticas de dança e meditação, para você descobrir e expressar a dança que já existe em você.</t>
+          <t>Workshops som integrerer bevissthet om bevegelse med praksiser innen dans og meditasjon, slik at du kan oppdage og uttrykke den dansen som allerede finnes i deg.</t>
         </is>
       </c>
       <c r="G646" s="6" t="inlineStr">
@@ -23791,7 +24043,11 @@
           <t>Completo (3 idiomas)</t>
         </is>
       </c>
-      <c r="H646" s="5" t="inlineStr"/>
+      <c r="H646" s="5" t="inlineStr">
+        <is>
+          <t>[EN: Translation was missing.] | [NO: Was not translated.]</t>
+        </is>
+      </c>
     </row>
     <row r="647">
       <c r="A647" s="7" t="n">
@@ -23850,12 +24106,12 @@
       </c>
       <c r="E648" s="5" t="inlineStr">
         <is>
-          <t>Descubra a dança que existe em você.</t>
+          <t>Discover the dance that exists within you.</t>
         </is>
       </c>
       <c r="F648" s="5" t="inlineStr">
         <is>
-          <t>Descubra a dança que existe em você.</t>
+          <t>Oppdag dansen som finnes i deg.</t>
         </is>
       </c>
       <c r="G648" s="6" t="inlineStr">
@@ -23863,7 +24119,11 @@
           <t>Completo (3 idiomas)</t>
         </is>
       </c>
-      <c r="H648" s="5" t="inlineStr"/>
+      <c r="H648" s="5" t="inlineStr">
+        <is>
+          <t>[EN: Translation was missing.] | [NO: Was not translated.]</t>
+        </is>
+      </c>
     </row>
     <row r="649">
       <c r="A649" s="7" t="n">
@@ -24951,12 +25211,12 @@
       </c>
       <c r="E676" s="5" t="inlineStr">
         <is>
-          <t>Biostretch é um sistema de exercícios...</t>
+          <t>Biostretch is an exercise system...</t>
         </is>
       </c>
       <c r="F676" s="5" t="inlineStr">
         <is>
-          <t>Biostretch é um sistema de exercícios...</t>
+          <t>Biostretch er et treningssystem...</t>
         </is>
       </c>
       <c r="G676" s="6" t="inlineStr">
@@ -24964,7 +25224,11 @@
           <t>Completo (3 idiomas)</t>
         </is>
       </c>
-      <c r="H676" s="5" t="inlineStr"/>
+      <c r="H676" s="5" t="inlineStr">
+        <is>
+          <t>[EN: Translation was missing.] | [NO: Was not translated.]</t>
+        </is>
+      </c>
     </row>
     <row r="677">
       <c r="A677" s="7" t="n">
@@ -26178,12 +26442,12 @@
       </c>
       <c r="E710" s="5" t="inlineStr">
         <is>
-          <t>Biostretch é um sistema de exercícios que promove a reconexão com o corpo por meio da consciência do movimento.</t>
+          <t>Biostretch is an exercise system that promotes reconnection with the body through movement awareness.</t>
         </is>
       </c>
       <c r="F710" s="5" t="inlineStr">
         <is>
-          <t>Biostretch é um sistema de exercícios que promove a reconexão com o corpo por meio da consciência do movimento.</t>
+          <t>Biostretch er et treningssystem som fremmer en gjenforening med kroppen gjennom bevissthet om bevegelse.</t>
         </is>
       </c>
       <c r="G710" s="6" t="inlineStr">
@@ -26191,7 +26455,11 @@
           <t>Completo (3 idiomas)</t>
         </is>
       </c>
-      <c r="H710" s="5" t="inlineStr"/>
+      <c r="H710" s="5" t="inlineStr">
+        <is>
+          <t>[EN: Translation was missing.] | [NO: Was not translated.]</t>
+        </is>
+      </c>
     </row>
     <row r="711">
       <c r="A711" s="7" t="n">
@@ -26214,12 +26482,12 @@
       </c>
       <c r="E711" s="10" t="inlineStr">
         <is>
-          <t>O método utiliza a atenção como sua principal ferramenta: um recurso simples, poderoso e acessível a todos. Ao direcioná-la para a experiência do movimento, ampliamos a percepção do corpo e abrimos espaço para novas possibilidades de organização corporal.</t>
+          <t>The method uses attention as its main tool: a simple, powerful resource accessible to everyone. By directing it to the experience of movement, we expand the perception of the body and open space for new possibilities of bodily organization.</t>
         </is>
       </c>
       <c r="F711" s="10" t="inlineStr">
         <is>
-          <t>O método utiliza a atenção como sua principal ferramenta: um recurso simples, poderoso e acessível a todos. Ao direcioná-la para a experiência do movimento, ampliamos a percepção do corpo e abrimos espaço para novas possibilidades de organização corporal.</t>
+          <t>Metoden bruker oppmerksomhet som sitt viktigste verktøy: en enkel, kraftfull ressurs som er tilgjengelig for alle. Ved å rette den mot bevegelsesopplevelsen, utvider vi oppfatningen av kroppen og åpner rom for nye muligheter for kroppslig organisering.</t>
         </is>
       </c>
       <c r="G711" s="11" t="inlineStr">
@@ -26227,7 +26495,11 @@
           <t>Completo (3 idiomas)</t>
         </is>
       </c>
-      <c r="H711" s="10" t="inlineStr"/>
+      <c r="H711" s="10" t="inlineStr">
+        <is>
+          <t>[EN: Translation was missing.] | [NO: Was not translated.]</t>
+        </is>
+      </c>
     </row>
     <row r="712">
       <c r="A712" s="2" t="n">
@@ -26250,12 +26522,12 @@
       </c>
       <c r="E712" s="5" t="inlineStr">
         <is>
-          <t>Inspirado em mais de quatro décadas de estudos em dança, Educação Somática e meditação, o método reconhece o corpo como um sistema inteligente, integrado e em constante transformação. Em vez de buscar desempenho ou correção, propõe uma investigação sutil da experiência corporal, na qual importa menos o que se faz e mais como se faz.</t>
+          <t>Inspired by more than four decades of studies in dance, Somatic Education, and meditation, the method recognizes the body as an intelligent, integrated system in constant transformation. Instead of seeking performance or correction, it proposes a subtle investigation of the bodily experience, where what is done matters less than how it is done.</t>
         </is>
       </c>
       <c r="F712" s="5" t="inlineStr">
         <is>
-          <t>Inspirado em mais de quatro décadas de estudos em dança, Educação Somática e meditação, o método reconhece o corpo como um sistema inteligente, integrado e em constante transformação. Em vez de buscar desempenho ou correção, propõe uma investigação sutil da experiência corporal, na qual importa menos o que se faz e mais como se faz.</t>
+          <t>Inspirert av over fire tiår med fordypning i dans, somatisk bevegelseslære og meditasjon, anerkjenner metoden kroppen som et intelligent, helhetlig system i kontinuerlig endring. I stedet for å jage etter prestasjon eller perfeksjon, inviterer den til en nennsom utforskning av den kroppslige opplevelsen – hvor det betyr mindre hva du gjør, og mer hvordan du gjør det.</t>
         </is>
       </c>
       <c r="G712" s="6" t="inlineStr">
@@ -26263,7 +26535,11 @@
           <t>Completo (3 idiomas)</t>
         </is>
       </c>
-      <c r="H712" s="5" t="inlineStr"/>
+      <c r="H712" s="5" t="inlineStr">
+        <is>
+          <t>[EN: Translation was missing.] | [NO: Oversatt fra portugisisk med poetisk og nyansert norsk (bokmål).]</t>
+        </is>
+      </c>
     </row>
     <row r="713">
       <c r="A713" s="7" t="n">
@@ -26286,12 +26562,12 @@
       </c>
       <c r="E713" s="10" t="inlineStr">
         <is>
-          <t>É dessa experiência de presença que nasce uma nova forma de perceber e habitar o corpo. Mas como essa transformação acontece na prática?</t>
+          <t>It is from this experience of presence that a new way of perceiving and inhabiting the body emerges. But how does this transformation happen in practice?</t>
         </is>
       </c>
       <c r="F713" s="10" t="inlineStr">
         <is>
-          <t>É dessa experiência de presença que nasce uma nova forma de perceber e habitar o corpo. Mas como essa transformação acontece na prática?</t>
+          <t>Det er ut fra denne opplevelsen av tilstedeværelse at en ny måte å sanse og bebo egen kropp på vokser frem. Men hvordan foregår egentlig denne forvandlingen i praksis?</t>
         </is>
       </c>
       <c r="G713" s="11" t="inlineStr">
@@ -26299,7 +26575,11 @@
           <t>Completo (3 idiomas)</t>
         </is>
       </c>
-      <c r="H713" s="10" t="inlineStr"/>
+      <c r="H713" s="10" t="inlineStr">
+        <is>
+          <t>[EN: Translated missing text with natural native flow.] | [NO: Oversatt fra portugisisk med naturlig idiomatisk klang.]</t>
+        </is>
+      </c>
     </row>
     <row r="714">
       <c r="A714" s="2" t="n">
@@ -26322,12 +26602,12 @@
       </c>
       <c r="E714" s="5" t="inlineStr">
         <is>
-          <t>O QUE É O BIOSTRETCH?</t>
+          <t>WHAT IS BIOSTRETCH?</t>
         </is>
       </c>
       <c r="F714" s="5" t="inlineStr">
         <is>
-          <t>O QUE É O BIOSTRETCH?</t>
+          <t>HVA ER BIOSTRETCH?</t>
         </is>
       </c>
       <c r="G714" s="6" t="inlineStr">
@@ -26335,7 +26615,11 @@
           <t>Completo (3 idiomas)</t>
         </is>
       </c>
-      <c r="H714" s="5" t="inlineStr"/>
+      <c r="H714" s="5" t="inlineStr">
+        <is>
+          <t>[EN: Translated section heading.] | [NO: Oversatt overskrift.]</t>
+        </is>
+      </c>
     </row>
     <row r="715">
       <c r="A715" s="7" t="n">
@@ -26358,12 +26642,12 @@
       </c>
       <c r="E715" s="10" t="inlineStr">
         <is>
-          <t>A prática do Biostretch convida você a desacelerar, relaxar o corpo e direcionar a atenção para movimentos simples e para as sensações que eles despertam.</t>
+          <t>The practice of Biostretch invites you to slow down, relax your body, and direct your attention to simple movements and the sensations they awaken.</t>
         </is>
       </c>
       <c r="F715" s="10" t="inlineStr">
         <is>
-          <t>A prática do Biostretch convida você a desacelerar, relaxar o corpo e direcionar a atenção para movimentos simples e para as sensações que eles despertam.</t>
+          <t>Biostretch inviterer deg til å gire ned, gi slipp på spenninger i kroppen og rette oppmerksomheten mot enkle bevegelser og følelsene de vekker.</t>
         </is>
       </c>
       <c r="G715" s="11" t="inlineStr">
@@ -26371,7 +26655,11 @@
           <t>Completo (3 idiomas)</t>
         </is>
       </c>
-      <c r="H715" s="10" t="inlineStr"/>
+      <c r="H715" s="10" t="inlineStr">
+        <is>
+          <t>[EN: Translation was missing.] | [NO: Oversatt med naturlige norske uttrykk for avspenning og bevissthet.]</t>
+        </is>
+      </c>
     </row>
     <row r="716">
       <c r="A716" s="2" t="n">
@@ -26394,12 +26682,12 @@
       </c>
       <c r="E716" s="5" t="inlineStr">
         <is>
-          <t>Nessa exploração, torna-se possível reconhecer padrões de tensão, hábitos de movimento e formas de organização corporal que costumam permanecer fora da nossa percepção por operarem de forma automática e inconsciente. A aparente simplicidade da prática revela um trabalho profundo de escuta, percepção e reorganização.</t>
+          <t>In this exploration, it becomes possible to recognize tension patterns, movement habits, and forms of bodily organization that usually remain outside our perception because they operate automatically and unconsciously. The apparent simplicity of the practice reveals a profound work of listening, perception, and reorganization.</t>
         </is>
       </c>
       <c r="F716" s="5" t="inlineStr">
         <is>
-          <t>Nessa exploração, torna-se possível reconhecer padrões de tensão, hábitos de movimento e formas de organização corporal que costumam permanecer fora da nossa percepção por operarem de forma automática e inconsciente. A aparente simplicidade da prática revela um trabalho profundo de escuta, percepção e reorganização.</t>
+          <t>Gjennom denne utforskningen blir det mulig å legge merke til spenningsmønstre, bevegelsesvaner og måter kroppen organiserer seg på, som vanligvis unnslipper oppmerksomheten vår fordi de foregår automatisk og ubevisst. Den tilsynelatende enkelheten i øvelsene åpner opp for en dyp prosess av lytting, sansing og kroppslig reorganisering.</t>
         </is>
       </c>
       <c r="G716" s="6" t="inlineStr">
@@ -26407,7 +26695,11 @@
           <t>Completo (3 idiomas)</t>
         </is>
       </c>
-      <c r="H716" s="5" t="inlineStr"/>
+      <c r="H716" s="5" t="inlineStr">
+        <is>
+          <t>[EN: Translation was missing.] | [NO: Oversatt med presise somatiske begreper på norsk.]</t>
+        </is>
+      </c>
     </row>
     <row r="717">
       <c r="A717" s="7" t="n">
@@ -26430,12 +26722,12 @@
       </c>
       <c r="E717" s="10" t="inlineStr">
         <is>
-          <t>Ao serem realizados de forma lenta, suave e sem esforço, os exercícios favorecem um estado de equilíbrio no sistema nervoso, responsável por coordenar a comunicação entre corpo e mente e regular as funções do organismo. Nesse estado, o corpo encontra espaço para liberar tensões, reorganizar-se e recuperar a fluidez natural do movimento.</t>
+          <t>When performed slowly, gently, and effortlessly, the exercises promote a state of balance in the nervous system, responsible for coordinating communication between body and mind and regulating bodily functions. In this state, the body finds space to release tension, reorganize itself, and recover the natural fluidity of movement.</t>
         </is>
       </c>
       <c r="F717" s="10" t="inlineStr">
         <is>
-          <t>Ao serem realizados de forma lenta, suave e sem esforço, os exercícios favorecem um estado de equilíbrio no sistema nervoso, responsável por coordenar a comunicação entre corpo e mente e regular as funções do organismo. Nesse estado, o corpo encontra espaço para liberar tensões, reorganizar-se e recuperar a fluidez natural do movimento.</t>
+          <t>Når bevegelsene utføres rolig, mykt og uten anstrengelse, stimuleres en tilstand av balanse i nervesystemet – bindeleddet som koordinerer samspillet mellom kropp og sinn og regulerer kroppens funksjoner. I denne modusen finner kroppen rom til å slippe tak i spenninger, finne tilbake til likevekt og gjenvinne en naturlig, fri bevegelsesflyt.</t>
         </is>
       </c>
       <c r="G717" s="11" t="inlineStr">
@@ -26443,7 +26735,11 @@
           <t>Completo (3 idiomas)</t>
         </is>
       </c>
-      <c r="H717" s="10" t="inlineStr"/>
+      <c r="H717" s="10" t="inlineStr">
+        <is>
+          <t>[EN: Translation was missing.] | [NO: Oversatt med flytende, fysiologisk korrekt norsk bokmål.]</t>
+        </is>
+      </c>
     </row>
     <row r="718">
       <c r="A718" s="2" t="n">
@@ -26466,12 +26762,12 @@
       </c>
       <c r="E718" s="5" t="inlineStr">
         <is>
-          <t>Mais do que ensinar novos movimentos, o Biostretch fortalece a confiança na inteligência inata do corpo e convida a redescobrir o prazer de mover-se com liberdade, presença e consciência. O melhor é que essa experiência está ao alcance de qualquer pessoa.</t>
+          <t>More than teaching new movements, Biostretch strengthens trust in the body's innate intelligence and invites you to rediscover the pleasure of moving with freedom, presence, and awareness. The best part is that this experience is within anyone's reach.</t>
         </is>
       </c>
       <c r="F718" s="5" t="inlineStr">
         <is>
-          <t>Mais do que ensinar novos movimentos, o Biostretch fortalece a confiança na inteligência inata do corpo e convida a redescobrir o prazer de mover-se com liberdade, presença e consciência. O melhor é que essa experiência está ao alcance de qualquer pessoa.</t>
+          <t>Mer enn å lære bort nye bevegelser, styrker Biostretch tilliten til kroppens medfødte intelligens og inviterer til å gjenoppdage gleden ved å bevege seg med frihet, tilstedeværelse og bevissthet. Det beste av alt er at denne opplevelsen er tilgjengelig for alle.</t>
         </is>
       </c>
       <c r="G718" s="6" t="inlineStr">
@@ -26479,7 +26775,11 @@
           <t>Completo (3 idiomas)</t>
         </is>
       </c>
-      <c r="H718" s="5" t="inlineStr"/>
+      <c r="H718" s="5" t="inlineStr">
+        <is>
+          <t>[EN: Translation was missing.] | [NO: Oversatt med varm, innbydende tone tilpasset dans og somatikk.]</t>
+        </is>
+      </c>
     </row>
     <row r="719">
       <c r="A719" s="7" t="n">
@@ -26502,12 +26802,12 @@
       </c>
       <c r="E719" s="10" t="inlineStr">
         <is>
-          <t>COMO ATUA?</t>
+          <t>HOW DOES IT WORK?</t>
         </is>
       </c>
       <c r="F719" s="10" t="inlineStr">
         <is>
-          <t>COMO ATUA?</t>
+          <t>HVORDAN FUNGERER DET?</t>
         </is>
       </c>
       <c r="G719" s="11" t="inlineStr">
@@ -26515,7 +26815,11 @@
           <t>Completo (3 idiomas)</t>
         </is>
       </c>
-      <c r="H719" s="10" t="inlineStr"/>
+      <c r="H719" s="10" t="inlineStr">
+        <is>
+          <t>[EN: Translation was missing.] | [NO: Oversatt overskrift med naturlig norsk ordlyd]</t>
+        </is>
+      </c>
     </row>
     <row r="720">
       <c r="A720" s="2" t="n">
@@ -26538,12 +26842,12 @@
       </c>
       <c r="E720" s="5" t="inlineStr">
         <is>
-          <t>O Biostretch pode ser praticado por pessoas de todas as idades e diferentes níveis de experiência, condicionamento físico ou mobilidade.</t>
+          <t>Biostretch can be practiced by people of all ages and different levels of experience, physical conditioning, or mobility.</t>
         </is>
       </c>
       <c r="F720" s="5" t="inlineStr">
         <is>
-          <t>O Biostretch pode ser praticado por pessoas de todas as idades e diferentes níveis de experiência, condicionamento físico ou mobilidade.</t>
+          <t>Biostretch passer for mennesker i alle aldre og med ulik erfaring, fysisk form eller bevegelighet.</t>
         </is>
       </c>
       <c r="G720" s="6" t="inlineStr">
@@ -26551,7 +26855,11 @@
           <t>Completo (3 idiomas)</t>
         </is>
       </c>
-      <c r="H720" s="5" t="inlineStr"/>
+      <c r="H720" s="5" t="inlineStr">
+        <is>
+          <t>[EN: Translation was missing.] | [NO: Oversatt med inkluderende, naturlig ordlyd.]</t>
+        </is>
+      </c>
     </row>
     <row r="721">
       <c r="A721" s="7" t="n">
@@ -26574,12 +26882,12 @@
       </c>
       <c r="E721" s="10" t="inlineStr">
         <is>
-          <t>A prática respeita a individualidade de cada corpo. Não existe um movimento ideal a ser alcançado nem um padrão externo a ser seguido. Cada pessoa explora as sequências dentro de seus próprios limites e possibilidades, no seu próprio ritmo.</t>
+          <t>The practice respects the individuality of each body. There is no ideal movement to be achieved, nor an external standard to be followed. Each person explores the sequences within their own limits and possibilities, at their own pace.</t>
         </is>
       </c>
       <c r="F721" s="10" t="inlineStr">
         <is>
-          <t>A prática respeita a individualidade de cada corpo. Não existe um movimento ideal a ser alcançado nem um padrão externo a ser seguido. Cada pessoa explora as sequências dentro de seus próprios limites e possibilidades, no seu próprio ritmo.</t>
+          <t>Praksisen respekterer hver enkelt kropps unike forutsetninger. Det finnes ingen fasit eller ideell bevegelse man må strekke seg etter, og ingen ytre mal å følge. Hver deltaker utforsker øvelsene ut fra sine egne grenser og muligheter, i sitt eget tempo.</t>
         </is>
       </c>
       <c r="G721" s="11" t="inlineStr">
@@ -26587,7 +26895,11 @@
           <t>Completo (3 idiomas)</t>
         </is>
       </c>
-      <c r="H721" s="10" t="inlineStr"/>
+      <c r="H721" s="10" t="inlineStr">
+        <is>
+          <t>[EN: Translation was missing.] | [NO: Oversatt med fokus på individuell tilpasning og naturlig norsk språkføring.]</t>
+        </is>
+      </c>
     </row>
     <row r="722">
       <c r="A722" s="2" t="n">
@@ -26610,12 +26922,12 @@
       </c>
       <c r="E722" s="5" t="inlineStr">
         <is>
-          <t>Em vez de adaptar o corpo a um modelo, o Biostretch valoriza aquilo que cada pessoa já possui: sua capacidade de perceber, aprender e encontrar caminhos mais confortáveis e funcionais para o movimento. Assim, a prática fortalece a autonomia, a confiança e o prazer de habitar o próprio corpo.</t>
+          <t>Instead of adapting the body to a model, Biostretch values what each person already has: their ability to perceive, learn, and find more comfortable and functional paths for movement. Thus, the practice strengthens autonomy, confidence, and the pleasure of inhabiting one's own body.</t>
         </is>
       </c>
       <c r="F722" s="5" t="inlineStr">
         <is>
-          <t>Em vez de adaptar o corpo a um modelo, o Biostretch valoriza aquilo que cada pessoa já possui: sua capacidade de perceber, aprender e encontrar caminhos mais confortáveis e funcionais para o movimento. Assim, a prática fortalece a autonomia, a confiança e o prazer de habitar o próprio corpo.</t>
+          <t>I stedet for å tvinge kroppen inn i en gitt form, bygger Biostretch på ressursene du allerede bærer i deg: evnen til å sanse, lære og finne mer behagelige og funksjonelle bevegelsesmønstre. Slik fremmer metoden autonomi, trygghet og gleden ved å finne seg til rette i egen kropp.</t>
         </is>
       </c>
       <c r="G722" s="6" t="inlineStr">
@@ -26623,7 +26935,11 @@
           <t>Completo (3 idiomas)</t>
         </is>
       </c>
-      <c r="H722" s="5" t="inlineStr"/>
+      <c r="H722" s="5" t="inlineStr">
+        <is>
+          <t>[EN: Translation was missing.] | [NO: Oversatt med naturlige vendinger for kroppslig tilstedeværelse.]</t>
+        </is>
+      </c>
     </row>
     <row r="723">
       <c r="A723" s="7" t="n">
@@ -26646,12 +26962,12 @@
       </c>
       <c r="E723" s="10" t="inlineStr">
         <is>
-          <t>E o que essa prática pode transformar no dia a dia?</t>
+          <t>And what can this practice transform in daily life?</t>
         </is>
       </c>
       <c r="F723" s="10" t="inlineStr">
         <is>
-          <t>E o que essa prática pode transformar no dia a dia?</t>
+          <t>Og hva kan denne praksisen tilføre hverdagen din?</t>
         </is>
       </c>
       <c r="G723" s="11" t="inlineStr">
@@ -26659,7 +26975,11 @@
           <t>Completo (3 idiomas)</t>
         </is>
       </c>
-      <c r="H723" s="10" t="inlineStr"/>
+      <c r="H723" s="10" t="inlineStr">
+        <is>
+          <t>[EN: Translation was missing.] | [NO: Oversatt med naturlig overgangsspørsmål.]</t>
+        </is>
+      </c>
     </row>
     <row r="724">
       <c r="A724" s="2" t="n">
@@ -26682,12 +27002,12 @@
       </c>
       <c r="E724" s="5" t="inlineStr">
         <is>
-          <t>QUEM PODE PRATICAR?</t>
+          <t>WHO CAN PRACTICE?</t>
         </is>
       </c>
       <c r="F724" s="5" t="inlineStr">
         <is>
-          <t>QUEM PODE PRATICAR?</t>
+          <t>HVEM KAN DELTA?</t>
         </is>
       </c>
       <c r="G724" s="6" t="inlineStr">
@@ -26695,7 +27015,11 @@
           <t>Completo (3 idiomas)</t>
         </is>
       </c>
-      <c r="H724" s="5" t="inlineStr"/>
+      <c r="H724" s="5" t="inlineStr">
+        <is>
+          <t>[EN: Translation was missing.] | [NO: Oversatt overskrift.]</t>
+        </is>
+      </c>
     </row>
     <row r="725">
       <c r="A725" s="7" t="n">
@@ -26718,12 +27042,12 @@
       </c>
       <c r="E725" s="10" t="inlineStr">
         <is>
-          <t>A prática regular do Biostretch contribui para aliviar tensões, ampliar a mobilidade, melhorar a postura e tornar os movimentos mais leves, coordenados e confortáveis. Com o tempo, o corpo recupera a fluidez e eficiência, tornando as atividades do dia a dia mais fáceis e prazerosas.</t>
+          <t>Regular practice of Biostretch helps to relieve tension, increase mobility, improve posture, and make movements lighter, coordinated, and comfortable. Over time, the body recovers fluidity and efficiency, making daily activities easier and more pleasant.</t>
         </is>
       </c>
       <c r="F725" s="10" t="inlineStr">
         <is>
-          <t>A prática regular do Biostretch contribui para aliviar tensões, ampliar a mobilidade, melhorar a postura e tornar os movimentos mais leves, coordenados e confortáveis. Com o tempo, o corpo recupera a fluidez e eficiência, tornando as atividades do dia a dia mais fáceis e prazerosas.</t>
+          <t>Regelmessig praksis av Biostretch bidrar til å løse opp spenninger, øke bevegeligheten, forbedre holdningen og gjøre bevegelsene lettere, mer samkjørte og behagelige. Over tid gjenvinner kroppen sin smidighet og funksjonalitet, slik at hverdagens gjøremål oppleves lettere og mer lystbetont.</t>
         </is>
       </c>
       <c r="G725" s="11" t="inlineStr">
@@ -26731,7 +27055,11 @@
           <t>Completo (3 idiomas)</t>
         </is>
       </c>
-      <c r="H725" s="10" t="inlineStr"/>
+      <c r="H725" s="10" t="inlineStr">
+        <is>
+          <t>[EN: Translation was missing.] | [NO: Oversatt helse- og bevegelsesfordeler med idiomatisk norsk.]</t>
+        </is>
+      </c>
     </row>
     <row r="726">
       <c r="A726" s="2" t="n">
@@ -26754,12 +27082,12 @@
       </c>
       <c r="E726" s="5" t="inlineStr">
         <is>
-          <t>Ao favorecer o equilíbrio do sistema nervoso, a prática também ajuda a reduzir os efeitos do estresse, melhorar a qualidade da respiração e aliviar dores e desconfortos associados à tensão muscular, especialmente em regiões como pescoço, ombros e costas. Além disso, contribui para prevenir lesões relacionadas a padrões repetitivos e ao uso excessivo do corpo.</t>
+          <t>By promoting balance in the nervous system, the practice also helps reduce the effects of stress, improve breathing quality, and relieve pain and discomfort associated with muscle tension, especially in areas like the neck, shoulders, and back. Additionally, it contributes to preventing injuries related to repetitive patterns and overuse of the body.</t>
         </is>
       </c>
       <c r="F726" s="5" t="inlineStr">
         <is>
-          <t>Ao favorecer o equilíbrio do sistema nervoso, a prática também ajuda a reduzir os efeitos do estresse, melhorar a qualidade da respiração e aliviar dores e desconfortos associados à tensão muscular, especialmente em regiões como pescoço, ombros e costas. Além disso, contribui para prevenir lesões relacionadas a padrões repetitivos e ao uso excessivo do corpo.</t>
+          <t>Ved å fremme balanse i nervesystemet bidrar praksisen også til å dempe stress, forbedre pustekvaliteten og lindre ubehag forbundet med muskelspenninger – særlig i nakke, skuldre og rygg. I tillegg virker den forebyggende mot belastningsskader forårsaket av ensformige bevegelsesmønstre og overbelastning.</t>
         </is>
       </c>
       <c r="G726" s="6" t="inlineStr">
@@ -26767,7 +27095,11 @@
           <t>Completo (3 idiomas)</t>
         </is>
       </c>
-      <c r="H726" s="5" t="inlineStr"/>
+      <c r="H726" s="5" t="inlineStr">
+        <is>
+          <t>[EN: Translation was missing.] | [NO: Oversatt med korrekte anatomiske og ergonomiske uttrykk på norsk.]</t>
+        </is>
+      </c>
     </row>
     <row r="727">
       <c r="A727" s="7" t="n">
@@ -26790,12 +27122,12 @@
       </c>
       <c r="E727" s="10" t="inlineStr">
         <is>
-          <t>Com o tempo, essas mudanças se estendem para além da prática e passam a fazer parte da maneira como nos movemos, percebemos e utilizamos o corpo no dia a dia.</t>
+          <t>Over time, these changes extend beyond the practice and become part of how we move, perceive, and use our bodies in everyday life.</t>
         </is>
       </c>
       <c r="F727" s="10" t="inlineStr">
         <is>
-          <t>Com o tempo, essas mudanças se estendem para além da prática e passam a fazer parte da maneira como nos movemos, percebemos e utilizamos o corpo no dia a dia.</t>
+          <t>Over tid forplanter disse endringene seg utover selve timene, og blir en naturlig del av hvordan vi beveger oss, sanser og bruker kroppen i det daglige.</t>
         </is>
       </c>
       <c r="G727" s="11" t="inlineStr">
@@ -26803,7 +27135,11 @@
           <t>Completo (3 idiomas)</t>
         </is>
       </c>
-      <c r="H727" s="10" t="inlineStr"/>
+      <c r="H727" s="10" t="inlineStr">
+        <is>
+          <t>[EN: Translation was missing.] | [NO: Oversatt med naturlig poetisk flyt.]</t>
+        </is>
+      </c>
     </row>
     <row r="728">
       <c r="A728" s="2" t="n">
@@ -26826,12 +27162,12 @@
       </c>
       <c r="E728" s="5" t="inlineStr">
         <is>
-          <t>QUAIS OS BENEFÍCIOS?</t>
+          <t>WHAT ARE THE BENEFITS?</t>
         </is>
       </c>
       <c r="F728" s="5" t="inlineStr">
         <is>
-          <t>QUAIS OS BENEFÍCIOS?</t>
+          <t>HVA ER FORDELENE?</t>
         </is>
       </c>
       <c r="G728" s="6" t="inlineStr">
@@ -26839,7 +27175,11 @@
           <t>Completo (3 idiomas)</t>
         </is>
       </c>
-      <c r="H728" s="5" t="inlineStr"/>
+      <c r="H728" s="5" t="inlineStr">
+        <is>
+          <t>[EN: Translation was missing.] | [NO: Oversatt overskrift.]</t>
+        </is>
+      </c>
     </row>
     <row r="729">
       <c r="A729" s="7" t="n">
@@ -27742,12 +28082,12 @@
       </c>
       <c r="E751" s="10" t="inlineStr">
         <is>
-          <t>Uma abordagem integrada para o corpo e o movimento.</t>
+          <t>An integrated approach to the body and movement.</t>
         </is>
       </c>
       <c r="F751" s="10" t="inlineStr">
         <is>
-          <t>Uma abordagem integrada para o corpo e o movimento.</t>
+          <t>En integrert tilnærming til kropp og bevegelse.</t>
         </is>
       </c>
       <c r="G751" s="11" t="inlineStr">
@@ -27755,7 +28095,11 @@
           <t>Completo (3 idiomas)</t>
         </is>
       </c>
-      <c r="H751" s="10" t="inlineStr"/>
+      <c r="H751" s="10" t="inlineStr">
+        <is>
+          <t>[EN: Translated missing subtitle.] | [NO: Was not translated.]</t>
+        </is>
+      </c>
     </row>
     <row r="752">
       <c r="A752" s="2" t="n">
@@ -27855,7 +28199,7 @@
       </c>
       <c r="F754" s="5" t="inlineStr">
         <is>
-          <t>Vi inviterer forskjellige tilretteleggere, praksiser og kunnskap for å skape opplevelser som kobler oss tilbake til denne intelligensen. Klasser, kurs, innlevelser og samlinger som utforsker bevegelse, berøring, pust, uttrykk og tilstedeværelse.</t>
+          <t>Vi inviterer forskjellige tilretteleggere, praksiser og kunnskap for å skape opplevelser som kobler oss tilbake til denne intelligensen. Klasser, kurs, opplevelser og samlinger som utforsker bevegelse, berøring, pust, uttrykk og tilstedeværelse.</t>
         </is>
       </c>
       <c r="G754" s="6" t="inlineStr">
@@ -27863,7 +28207,11 @@
           <t>Completo (3 idiomas)</t>
         </is>
       </c>
-      <c r="H754" s="5" t="inlineStr"/>
+      <c r="H754" s="5" t="inlineStr">
+        <is>
+          <t>[NO: 'innlevelser' is not correct for 'vivências', 'opplevelser' is much more natural.]</t>
+        </is>
+      </c>
     </row>
     <row r="755">
       <c r="A755" s="7" t="n">
@@ -27999,7 +28347,7 @@
       </c>
       <c r="F758" s="5" t="inlineStr">
         <is>
-          <t>"Gjennom kroppen forbereder vi oss på å gå videre."</t>
+          <t>"Gjennom kroppen forbereder vi oss på å gå utover det kjente."</t>
         </is>
       </c>
       <c r="G758" s="6" t="inlineStr">
@@ -28007,7 +28355,11 @@
           <t>Completo (3 idiomas)</t>
         </is>
       </c>
-      <c r="H758" s="5" t="inlineStr"/>
+      <c r="H758" s="5" t="inlineStr">
+        <is>
+          <t>[NO: 'å gå videre' means 'move on'. 'ir além' means 'go beyond'. 'å gå utover det kjente' captures the poetic nuance.]</t>
+        </is>
+      </c>
     </row>
     <row r="759">
       <c r="A759" s="7" t="n">
@@ -28450,12 +28802,12 @@
       </c>
       <c r="E771" s="10" t="inlineStr">
         <is>
-          <t>Movement is raw material. From dance choreography is born, from silence the gesture is born, from the encounter the work is born. Art is what happens when the body has the freedom to express itself.</t>
+          <t>Movement is raw material. From dance, choreography is born; from silence, the gesture is born; from the encounter, the work is born. Art is what happens when the body has the freedom to express itself.</t>
         </is>
       </c>
       <c r="F771" s="10" t="inlineStr">
         <is>
-          <t>Bevegelse er råmateriale. Fra dans blir koreografi født, fra stillhet blir gesten født, fra møtet blir verket født. Kunst er det som skjer når kroppen har frihet til å uttrykke seg.</t>
+          <t>Bevegelse er råmateriale. Fra dansen fødes koreografien, fra stillheten fødes gesten, fra møtet fødes verket. Kunst er det som skjer når kroppen har frihet til å uttrykke seg.</t>
         </is>
       </c>
       <c r="G771" s="11" t="inlineStr">
@@ -28463,7 +28815,11 @@
           <t>Completo (3 idiomas)</t>
         </is>
       </c>
-      <c r="H771" s="10" t="inlineStr"/>
+      <c r="H771" s="10" t="inlineStr">
+        <is>
+          <t>[EN: Punctuated for better flow and poetic rhythm in English.] | [NO: Passive form 'fødes' sounds more poetic and natural than 'blir født' here.]</t>
+        </is>
+      </c>
     </row>
     <row r="772">
       <c r="A772" s="2" t="n">
@@ -28959,7 +29315,7 @@
       </c>
       <c r="F785" s="10" t="inlineStr">
         <is>
-          <t>Hvert møte er en del av en samtale kroppen bygger med seg selv.</t>
+          <t>Hvert møte er en del av en samtale kroppen fører med seg selv.</t>
         </is>
       </c>
       <c r="G785" s="11" t="inlineStr">
@@ -28967,7 +29323,11 @@
           <t>Completo (3 idiomas)</t>
         </is>
       </c>
-      <c r="H785" s="10" t="inlineStr"/>
+      <c r="H785" s="10" t="inlineStr">
+        <is>
+          <t>[NO: 'fører en samtale' is the natural Bokmål idiom, not 'bygger en samtale'.]</t>
+        </is>
+      </c>
     </row>
     <row r="786">
       <c r="A786" s="2" t="n">
@@ -29538,7 +29898,7 @@
       </c>
       <c r="F801" s="10" t="inlineStr">
         <is>
-          <t>Din Uttalelse / Opplevelse</t>
+          <t>Din Omtale / Opplevelse</t>
         </is>
       </c>
       <c r="G801" s="11" t="inlineStr">
@@ -29546,7 +29906,11 @@
           <t>Completo (3 idiomas)</t>
         </is>
       </c>
-      <c r="H801" s="10" t="inlineStr"/>
+      <c r="H801" s="10" t="inlineStr">
+        <is>
+          <t>[NO: 'Uttalelse' is usually formal/legal (statement). 'Omtale' or 'Tilbakemelding' is better for a review.]</t>
+        </is>
+      </c>
     </row>
     <row r="802">
       <c r="A802" s="2" t="n">
@@ -29862,7 +30226,7 @@
       </c>
       <c r="F810" s="5" t="inlineStr">
         <is>
-          <t>Transformativt &amp; Uforglemmelig</t>
+          <t>Transformerende &amp; Uforglemmelig</t>
         </is>
       </c>
       <c r="G810" s="6" t="inlineStr">
@@ -29870,7 +30234,11 @@
           <t>Completo (3 idiomas)</t>
         </is>
       </c>
-      <c r="H810" s="5" t="inlineStr"/>
+      <c r="H810" s="5" t="inlineStr">
+        <is>
+          <t>[NO: 'Transformerende' is the standard Bokmål form.]</t>
+        </is>
+      </c>
     </row>
     <row r="811">
       <c r="A811" s="7" t="n">
@@ -30330,7 +30698,7 @@
       </c>
       <c r="F823" s="10" t="inlineStr">
         <is>
-          <t>Gamle Oslo er et nabolag fylt av kontraster — mangfold, historie og kulturell rikdom eksisterer side om side med ulikhet i tilgang til kvalitetstjenester og aktiviteter. Det er nettopp denne sammenhengen som kaller oss til handling.</t>
+          <t>Gamle Oslo er et nabolag fylt av kontraster — mangfold, historie og kulturell rikdom eksisterer side om side med ulikhet i tilgang til kvalitetstjenester og aktiviteter. Det er nettopp denne virkeligheten som kaller oss til handling.</t>
         </is>
       </c>
       <c r="G823" s="11" t="inlineStr">
@@ -30338,7 +30706,11 @@
           <t>Completo (3 idiomas)</t>
         </is>
       </c>
-      <c r="H823" s="10" t="inlineStr"/>
+      <c r="H823" s="10" t="inlineStr">
+        <is>
+          <t>[NO: Literal translation of 'contexto'. 'virkeligheten' makes much more sense idiomatically.]</t>
+        </is>
+      </c>
     </row>
     <row r="824">
       <c r="A824" s="2" t="n">
@@ -30366,7 +30738,7 @@
       </c>
       <c r="F824" s="5" t="inlineStr">
         <is>
-          <t>Dance2Dance fødes i dette territoriet med et tydelig oppdrag: at dans, kroppsuttrykk og velvtære ikke skal være et privilegium for dem som kan betale. Hvert workshop vi utvikler har samme kvalitet, samme omsorg og samme intensjon — uavhengig av hvem som er i rommet.</t>
+          <t>Dance2Dance fødes i dette territoriet med et tydelig oppdrag: at dans, kroppsuttrykk og velvære ikke skal være et privilegium for dem som kan betale. Hver workshop vi utvikler har samme kvalitet, samme omsorg og samme intensjon — uavhengig av hvem som er i rommet.</t>
         </is>
       </c>
       <c r="G824" s="6" t="inlineStr">
@@ -30374,7 +30746,11 @@
           <t>Completo (3 idiomas)</t>
         </is>
       </c>
-      <c r="H824" s="5" t="inlineStr"/>
+      <c r="H824" s="5" t="inlineStr">
+        <is>
+          <t>[NO: Typos fixed: 'velvtære' -&gt; 'velvære'. 'Hvert' -&gt; 'Hver' (workshop is masculine/feminine, not neuter).]</t>
+        </is>
+      </c>
     </row>
     <row r="825">
       <c r="A825" s="7" t="n">
@@ -30726,7 +31102,7 @@
       </c>
       <c r="F834" s="5" t="inlineStr">
         <is>
-          <t>En modell for universell tilgang til kultur og bevegelse. Premium workshops, gratis for beboere i Gamle Oslo — bæret av flere finansieringskilder.</t>
+          <t>En modell for universell tilgang til kultur og bevegelse. Premium workshops, gratis for beboere i Gamle Oslo — båret av flere finansieringskilder.</t>
         </is>
       </c>
       <c r="G834" s="6" t="inlineStr">
@@ -30734,7 +31110,11 @@
           <t>Completo (3 idiomas)</t>
         </is>
       </c>
-      <c r="H834" s="5" t="inlineStr"/>
+      <c r="H834" s="5" t="inlineStr">
+        <is>
+          <t>[NO: 'bæret' is incorrect conjugation, should be 'båret'.]</t>
+        </is>
+      </c>
     </row>
     <row r="835">
       <c r="A835" s="7" t="n">
@@ -30870,7 +31250,7 @@
       </c>
       <c r="F838" s="5" t="inlineStr">
         <is>
-          <t>Dance2Dance er designet for å ikke støle på en enkelt kilde. Vår bærekraft kommer fra den strategiske kombinasjonen av flere pilarer — hver enkelt essensiell, ingen tilstrekkelig alene.</t>
+          <t>Dance2Dance er designet for å ikke stole på en enkelt kilde. Vår bærekraft kommer fra den strategiske kombinasjonen av flere pilarer — hver enkelt essensiell, ingen tilstrekkelig alene.</t>
         </is>
       </c>
       <c r="G838" s="6" t="inlineStr">
@@ -30878,7 +31258,11 @@
           <t>Completo (3 idiomas)</t>
         </is>
       </c>
-      <c r="H838" s="5" t="inlineStr"/>
+      <c r="H838" s="5" t="inlineStr">
+        <is>
+          <t>[NO: Typo: 'støle' -&gt; 'stole' (rely on).]</t>
+        </is>
+      </c>
     </row>
     <row r="839">
       <c r="A839" s="7" t="n">
@@ -31698,7 +32082,7 @@
       </c>
       <c r="F861" s="10" t="inlineStr">
         <is>
-          <t>De som mottar det gratis, mottar nøyaktig det samme som de som betaler. Vi gjør den reelle prisen synlig fordi opplevd verdi betyr noe — for støttespillere og deltakere alike.</t>
+          <t>De som mottar det gratis, mottar nøyaktig det samme som de som betaler. Vi gjør den reelle prisen synlig fordi opplevd verdi betyr noe — både for støttespillere og deltakere.</t>
         </is>
       </c>
       <c r="G861" s="11" t="inlineStr">
@@ -31706,7 +32090,11 @@
           <t>Completo (3 idiomas)</t>
         </is>
       </c>
-      <c r="H861" s="10" t="inlineStr"/>
+      <c r="H861" s="10" t="inlineStr">
+        <is>
+          <t>[NO: Used English word 'alike'. Changed to 'både for... og...' (both for... and...).]</t>
+        </is>
+      </c>
     </row>
     <row r="862">
       <c r="A862" s="2" t="n">
@@ -32418,7 +32806,7 @@
       </c>
       <c r="F881" s="10" t="inlineStr">
         <is>
-          <t>Investorer unngår prosjekter som er avhengige av én enkelt donor. Dance2Dance ble bygget på 4 inntekts-pilarer som garanterer lang levetid, økonomisk sikkerhet og risikoreduksjon for alle interessenter.</t>
+          <t>Investorer unngår prosjekter som er avhengige av én enkelt donor. Dance2Dance ble bygget på 4 inntektspilarer som garanterer lang levetid, økonomisk sikkerhet og risikoreduksjon for alle interessenter.</t>
         </is>
       </c>
       <c r="G881" s="11" t="inlineStr">
@@ -32426,7 +32814,11 @@
           <t>Completo (3 idiomas)</t>
         </is>
       </c>
-      <c r="H881" s="10" t="inlineStr"/>
+      <c r="H881" s="10" t="inlineStr">
+        <is>
+          <t>[NO: Norwegian uses closed compounds: 'inntekts-pilarer' -&gt; 'inntektspilarer'.]</t>
+        </is>
+      </c>
     </row>
     <row r="882">
       <c r="A882" s="2" t="n">
@@ -33246,7 +33638,7 @@
       </c>
       <c r="F904" s="5" t="inlineStr">
         <is>
-          <t>Våre gratis plasser er ikke veldedighet, de er fullstendige stipender finansiert av vårt økosystem. Ved å prise workshopen for eksterne deltakere, beviser vi den høye verdien levert til lokale innbyggere og våre investorer.</t>
+          <t>Våre gratis plasser er ikke veldedighet, de er fullfinansierte stipender finansiert av vårt økosystem. Ved å prise workshopen for eksterne deltakere, beviser vi den høye verdien som leveres til lokale innbyggere og våre investorer.</t>
         </is>
       </c>
       <c r="G904" s="6" t="inlineStr">
@@ -33254,7 +33646,11 @@
           <t>Completo (3 idiomas)</t>
         </is>
       </c>
-      <c r="H904" s="5" t="inlineStr"/>
+      <c r="H904" s="5" t="inlineStr">
+        <is>
+          <t>[NO: Corrected phrasing: 'fullstendige stipender' to 'fullfinansierte stipender'. 'verdien levert til' to 'verdien som leveres til'.]</t>
+        </is>
+      </c>
     </row>
     <row r="905">
       <c r="A905" s="7" t="n">

</xml_diff>